<commit_message>
Recalibrate Rio targets (DAMA > CAB) and fix Excel % formatting
- Targets proportional to sales mix: CAB 2596, DAMA 2703, KIDS 2751
- Talla sheet: integer % display (18%, 25%, etc.)
- Color sheet: decimal % display (20.11%, 12.78%, etc.)

Co-authored-by: scm-svg <scm-svg@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/RIO_ORIGINAL_Proyeccion_Produccion.xlsx
+++ b/RIO_ORIGINAL_Proyeccion_Produccion.xlsx
@@ -55,7 +55,7 @@
     <t>• Tela Jabón Microfibra: consumo en kg/und (CAB 0.5 · DAMA 0.4 · KIDS 0.26).</t>
   </si>
   <si>
-    <t>• Meta de producción: CAB 2,650 · DAMA 2,450 · KIDS 2,950 und (mínimo compromiso).</t>
+    <t>• Meta de producción: CAB 2,596 · DAMA 2,703 · KIDS 2,751 und (mínimo compromiso).</t>
   </si>
   <si>
     <t>• CAB: sin 3XL ni 4XL en producción; 2XL con boost moderado (+22%).</t>
@@ -553,7 +553,7 @@
     <t>4. CANTIDAD A PRODUCIR</t>
   </si>
   <si>
-    <t>• Metas MÍN: CAB 2,650 · DAMA 2,450 · KIDS 2,950 und.</t>
+    <t>• Metas MÍN: CAB 2,596 · DAMA 2,703 · KIDS 2,751 und.</t>
   </si>
   <si>
     <t>• Color: % sobre ventas históricas Oct–Ago; talla: % sobre ventas Jun–Ago.</t>
@@ -587,11 +587,12 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="4">
-    <numFmt numFmtId="164" formatCode="0.0%"/>
+  <numFmts count="5">
+    <numFmt numFmtId="164" formatCode="0%"/>
     <numFmt numFmtId="165" formatCode="0.0"/>
-    <numFmt numFmtId="166" formatCode="0.0000"/>
+    <numFmt numFmtId="166" formatCode="0.0000%"/>
     <numFmt numFmtId="167" formatCode="#,##0"/>
+    <numFmt numFmtId="168" formatCode="0.00%"/>
   </numFmts>
   <fonts count="5">
     <font>
@@ -690,7 +691,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -705,6 +706,7 @@
     <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="167" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1383,7 +1385,7 @@
         <v>37</v>
       </c>
       <c r="B38" s="10">
-        <v>2650</v>
+        <v>2596</v>
       </c>
     </row>
     <row r="39" spans="1:6">
@@ -1391,7 +1393,7 @@
         <v>38</v>
       </c>
       <c r="B39" s="10">
-        <v>2838</v>
+        <v>2782</v>
       </c>
     </row>
     <row r="40" spans="1:6">
@@ -1631,7 +1633,7 @@
         <v>37</v>
       </c>
       <c r="B62" s="10">
-        <v>2450</v>
+        <v>2703</v>
       </c>
     </row>
     <row r="63" spans="1:6">
@@ -1639,7 +1641,7 @@
         <v>38</v>
       </c>
       <c r="B63" s="10">
-        <v>2628</v>
+        <v>2893</v>
       </c>
     </row>
     <row r="64" spans="1:6">
@@ -1879,7 +1881,7 @@
         <v>37</v>
       </c>
       <c r="B86" s="10">
-        <v>2950</v>
+        <v>2751</v>
       </c>
     </row>
     <row r="87" spans="1:6">
@@ -1887,7 +1889,7 @@
         <v>38</v>
       </c>
       <c r="B87" s="10">
-        <v>3165</v>
+        <v>2952</v>
       </c>
     </row>
     <row r="88" spans="1:6">
@@ -1944,10 +1946,10 @@
         <v>1601</v>
       </c>
       <c r="E92">
-        <v>2650</v>
+        <v>2596</v>
       </c>
       <c r="F92">
-        <v>2838</v>
+        <v>2782</v>
       </c>
     </row>
     <row r="93" spans="1:6">
@@ -1964,10 +1966,10 @@
         <v>1462</v>
       </c>
       <c r="E93">
-        <v>2450</v>
+        <v>2703</v>
       </c>
       <c r="F93">
-        <v>2628</v>
+        <v>2893</v>
       </c>
     </row>
     <row r="94" spans="1:6">
@@ -1984,10 +1986,10 @@
         <v>2866</v>
       </c>
       <c r="E94">
-        <v>2950</v>
+        <v>2751</v>
       </c>
       <c r="F94">
-        <v>3165</v>
+        <v>2952</v>
       </c>
     </row>
     <row r="95" spans="1:6">
@@ -2007,7 +2009,7 @@
         <v>8050</v>
       </c>
       <c r="F95" s="11">
-        <v>8631</v>
+        <v>8627</v>
       </c>
     </row>
     <row r="97" spans="1:6">
@@ -2271,84 +2273,84 @@
       <c r="A5" t="s">
         <v>72</v>
       </c>
-      <c r="B5" s="8">
-        <v>0.176</v>
+      <c r="B5" s="5">
+        <v>0.18</v>
       </c>
       <c r="C5" s="9">
-        <v>466</v>
+        <v>458</v>
       </c>
       <c r="D5" s="9">
-        <v>501</v>
+        <v>493</v>
       </c>
     </row>
     <row r="6" spans="1:4">
       <c r="A6" t="s">
         <v>73</v>
       </c>
-      <c r="B6" s="8">
+      <c r="B6" s="5">
         <v>0.25</v>
       </c>
       <c r="C6" s="9">
-        <v>663</v>
+        <v>648</v>
       </c>
       <c r="D6" s="9">
-        <v>708</v>
+        <v>691</v>
       </c>
     </row>
     <row r="7" spans="1:4">
       <c r="A7" t="s">
         <v>74</v>
       </c>
-      <c r="B7" s="8">
-        <v>0.274</v>
+      <c r="B7" s="5">
+        <v>0.27</v>
       </c>
       <c r="C7" s="9">
-        <v>726</v>
+        <v>710</v>
       </c>
       <c r="D7" s="9">
-        <v>775</v>
+        <v>759</v>
       </c>
     </row>
     <row r="8" spans="1:4">
       <c r="A8" t="s">
         <v>75</v>
       </c>
-      <c r="B8" s="8">
-        <v>0.218</v>
+      <c r="B8" s="5">
+        <v>0.22</v>
       </c>
       <c r="C8" s="9">
-        <v>578</v>
+        <v>569</v>
       </c>
       <c r="D8" s="9">
-        <v>618</v>
+        <v>609</v>
       </c>
     </row>
     <row r="9" spans="1:4">
       <c r="A9" t="s">
         <v>76</v>
       </c>
-      <c r="B9" s="8">
-        <v>0.08199999999999999</v>
+      <c r="B9" s="5">
+        <v>0.08</v>
       </c>
       <c r="C9" s="9">
-        <v>217</v>
+        <v>211</v>
       </c>
       <c r="D9" s="9">
-        <v>236</v>
+        <v>230</v>
       </c>
     </row>
     <row r="10" spans="1:4">
       <c r="A10" s="4" t="s">
         <v>77</v>
       </c>
-      <c r="B10" s="8">
+      <c r="B10" s="5">
         <v>1</v>
       </c>
       <c r="C10" s="9">
-        <v>2650</v>
+        <v>2596</v>
       </c>
       <c r="D10" s="9">
-        <v>2838</v>
+        <v>2782</v>
       </c>
     </row>
     <row r="12" spans="1:4">
@@ -2374,84 +2376,84 @@
       <c r="A14" t="s">
         <v>79</v>
       </c>
-      <c r="B14" s="8">
+      <c r="B14" s="5">
         <v>0.21</v>
       </c>
       <c r="C14" s="9">
-        <v>514</v>
+        <v>566</v>
       </c>
       <c r="D14" s="9">
-        <v>552</v>
+        <v>605</v>
       </c>
     </row>
     <row r="15" spans="1:4">
       <c r="A15" t="s">
         <v>72</v>
       </c>
-      <c r="B15" s="8">
+      <c r="B15" s="5">
         <v>0.29</v>
       </c>
       <c r="C15" s="9">
-        <v>711</v>
+        <v>787</v>
       </c>
       <c r="D15" s="9">
-        <v>759</v>
+        <v>841</v>
       </c>
     </row>
     <row r="16" spans="1:4">
       <c r="A16" t="s">
         <v>73</v>
       </c>
-      <c r="B16" s="8">
-        <v>0.242</v>
+      <c r="B16" s="5">
+        <v>0.24</v>
       </c>
       <c r="C16" s="9">
-        <v>594</v>
+        <v>654</v>
       </c>
       <c r="D16" s="9">
-        <v>636</v>
+        <v>698</v>
       </c>
     </row>
     <row r="17" spans="1:4">
       <c r="A17" t="s">
         <v>74</v>
       </c>
-      <c r="B17" s="8">
-        <v>0.153</v>
+      <c r="B17" s="5">
+        <v>0.15</v>
       </c>
       <c r="C17" s="9">
-        <v>376</v>
+        <v>414</v>
       </c>
       <c r="D17" s="9">
-        <v>405</v>
+        <v>445</v>
       </c>
     </row>
     <row r="18" spans="1:4">
       <c r="A18" t="s">
         <v>75</v>
       </c>
-      <c r="B18" s="8">
-        <v>0.104</v>
+      <c r="B18" s="5">
+        <v>0.1</v>
       </c>
       <c r="C18" s="9">
-        <v>255</v>
+        <v>282</v>
       </c>
       <c r="D18" s="9">
-        <v>276</v>
+        <v>304</v>
       </c>
     </row>
     <row r="19" spans="1:4">
       <c r="A19" s="4" t="s">
         <v>77</v>
       </c>
-      <c r="B19" s="8">
+      <c r="B19" s="5">
         <v>1</v>
       </c>
       <c r="C19" s="9">
-        <v>2450</v>
+        <v>2703</v>
       </c>
       <c r="D19" s="9">
-        <v>2628</v>
+        <v>2893</v>
       </c>
     </row>
     <row r="21" spans="1:4">
@@ -2477,112 +2479,112 @@
       <c r="A23" t="s">
         <v>81</v>
       </c>
-      <c r="B23" s="8">
-        <v>0.156</v>
+      <c r="B23" s="5">
+        <v>0.16</v>
       </c>
       <c r="C23" s="9">
-        <v>460</v>
+        <v>430</v>
       </c>
       <c r="D23" s="9">
-        <v>493</v>
+        <v>461</v>
       </c>
     </row>
     <row r="24" spans="1:4">
       <c r="A24" t="s">
         <v>82</v>
       </c>
-      <c r="B24" s="8">
-        <v>0.161</v>
+      <c r="B24" s="5">
+        <v>0.16</v>
       </c>
       <c r="C24" s="9">
-        <v>474</v>
+        <v>441</v>
       </c>
       <c r="D24" s="9">
-        <v>507</v>
+        <v>473</v>
       </c>
     </row>
     <row r="25" spans="1:4">
       <c r="A25" t="s">
         <v>83</v>
       </c>
-      <c r="B25" s="8">
-        <v>0.139</v>
+      <c r="B25" s="5">
+        <v>0.14</v>
       </c>
       <c r="C25" s="9">
-        <v>410</v>
+        <v>382</v>
       </c>
       <c r="D25" s="9">
-        <v>440</v>
+        <v>411</v>
       </c>
     </row>
     <row r="26" spans="1:4">
       <c r="A26" t="s">
         <v>84</v>
       </c>
-      <c r="B26" s="8">
-        <v>0.139</v>
+      <c r="B26" s="5">
+        <v>0.14</v>
       </c>
       <c r="C26" s="9">
-        <v>410</v>
+        <v>384</v>
       </c>
       <c r="D26" s="9">
-        <v>441</v>
+        <v>412</v>
       </c>
     </row>
     <row r="27" spans="1:4">
       <c r="A27" t="s">
         <v>85</v>
       </c>
-      <c r="B27" s="8">
-        <v>0.134</v>
+      <c r="B27" s="5">
+        <v>0.13</v>
       </c>
       <c r="C27" s="9">
-        <v>394</v>
+        <v>367</v>
       </c>
       <c r="D27" s="9">
-        <v>422</v>
+        <v>393</v>
       </c>
     </row>
     <row r="28" spans="1:4">
       <c r="A28" t="s">
         <v>86</v>
       </c>
-      <c r="B28" s="8">
-        <v>0.154</v>
+      <c r="B28" s="5">
+        <v>0.15</v>
       </c>
       <c r="C28" s="9">
-        <v>454</v>
+        <v>424</v>
       </c>
       <c r="D28" s="9">
-        <v>487</v>
+        <v>455</v>
       </c>
     </row>
     <row r="29" spans="1:4">
       <c r="A29" t="s">
         <v>87</v>
       </c>
-      <c r="B29" s="8">
-        <v>0.118</v>
+      <c r="B29" s="5">
+        <v>0.12</v>
       </c>
       <c r="C29" s="9">
-        <v>348</v>
+        <v>323</v>
       </c>
       <c r="D29" s="9">
-        <v>375</v>
+        <v>347</v>
       </c>
     </row>
     <row r="30" spans="1:4">
       <c r="A30" s="4" t="s">
         <v>77</v>
       </c>
-      <c r="B30" s="8">
+      <c r="B30" s="5">
         <v>1</v>
       </c>
       <c r="C30" s="9">
-        <v>2950</v>
+        <v>2751</v>
       </c>
       <c r="D30" s="9">
-        <v>3165</v>
+        <v>2952</v>
       </c>
     </row>
   </sheetData>
@@ -2623,148 +2625,148 @@
       <c r="A5" t="s">
         <v>91</v>
       </c>
-      <c r="B5" s="8">
-        <v>0.2011320754716981</v>
+      <c r="B5" s="12">
+        <v>0.2014637904468413</v>
       </c>
       <c r="C5" s="9">
-        <v>533</v>
+        <v>523</v>
       </c>
       <c r="D5" s="9">
-        <v>568</v>
+        <v>557</v>
       </c>
     </row>
     <row r="6" spans="1:4">
       <c r="A6" t="s">
         <v>92</v>
       </c>
-      <c r="B6" s="8">
-        <v>0.1283018867924528</v>
+      <c r="B6" s="12">
+        <v>0.1278890600924499</v>
       </c>
       <c r="C6" s="9">
-        <v>340</v>
+        <v>332</v>
       </c>
       <c r="D6" s="9">
-        <v>364</v>
+        <v>356</v>
       </c>
     </row>
     <row r="7" spans="1:4">
       <c r="A7" t="s">
         <v>93</v>
       </c>
-      <c r="B7" s="8">
-        <v>0.1207547169811321</v>
+      <c r="B7" s="12">
+        <v>0.1209553158705701</v>
       </c>
       <c r="C7" s="9">
-        <v>320</v>
+        <v>314</v>
       </c>
       <c r="D7" s="9">
-        <v>342</v>
+        <v>336</v>
       </c>
     </row>
     <row r="8" spans="1:4">
       <c r="A8" t="s">
         <v>94</v>
       </c>
-      <c r="B8" s="8">
-        <v>0.100377358490566</v>
+      <c r="B8" s="12">
+        <v>0.09976887519260401</v>
       </c>
       <c r="C8" s="9">
-        <v>266</v>
+        <v>259</v>
       </c>
       <c r="D8" s="9">
-        <v>284</v>
+        <v>277</v>
       </c>
     </row>
     <row r="9" spans="1:4">
       <c r="A9" t="s">
         <v>95</v>
       </c>
-      <c r="B9" s="8">
-        <v>0.09622641509433963</v>
+      <c r="B9" s="12">
+        <v>0.09591679506933744</v>
       </c>
       <c r="C9" s="9">
-        <v>255</v>
+        <v>249</v>
       </c>
       <c r="D9" s="9">
-        <v>273</v>
+        <v>267</v>
       </c>
     </row>
     <row r="10" spans="1:4">
       <c r="A10" t="s">
         <v>96</v>
       </c>
-      <c r="B10" s="8">
-        <v>0.0879245283018868</v>
+      <c r="B10" s="12">
+        <v>0.08782742681047766</v>
       </c>
       <c r="C10" s="9">
-        <v>233</v>
+        <v>228</v>
       </c>
       <c r="D10" s="9">
-        <v>250</v>
+        <v>245</v>
       </c>
     </row>
     <row r="11" spans="1:4">
       <c r="A11" t="s">
         <v>97</v>
       </c>
-      <c r="B11" s="8">
-        <v>0.08150943396226415</v>
+      <c r="B11" s="12">
+        <v>0.08166409861325115</v>
       </c>
       <c r="C11" s="9">
-        <v>216</v>
+        <v>212</v>
       </c>
       <c r="D11" s="9">
-        <v>231</v>
+        <v>227</v>
       </c>
     </row>
     <row r="12" spans="1:4">
       <c r="A12" t="s">
         <v>98</v>
       </c>
-      <c r="B12" s="8">
-        <v>0.06566037735849056</v>
+      <c r="B12" s="12">
+        <v>0.06548536209553159</v>
       </c>
       <c r="C12" s="9">
-        <v>174</v>
+        <v>170</v>
       </c>
       <c r="D12" s="9">
-        <v>187</v>
+        <v>183</v>
       </c>
     </row>
     <row r="13" spans="1:4">
       <c r="A13" t="s">
         <v>99</v>
       </c>
-      <c r="B13" s="8">
-        <v>0.05509433962264151</v>
+      <c r="B13" s="12">
+        <v>0.05508474576271186</v>
       </c>
       <c r="C13" s="9">
-        <v>146</v>
+        <v>143</v>
       </c>
       <c r="D13" s="9">
-        <v>158</v>
+        <v>154</v>
       </c>
     </row>
     <row r="14" spans="1:4">
       <c r="A14" t="s">
         <v>100</v>
       </c>
-      <c r="B14" s="8">
-        <v>0.04716981132075472</v>
+      <c r="B14" s="12">
+        <v>0.04776579352850539</v>
       </c>
       <c r="C14" s="9">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="D14" s="9">
-        <v>134</v>
+        <v>133</v>
       </c>
     </row>
     <row r="15" spans="1:4">
       <c r="A15" t="s">
         <v>101</v>
       </c>
-      <c r="B15" s="8">
-        <v>0.01584905660377358</v>
+      <c r="B15" s="12">
+        <v>0.01617873651771957</v>
       </c>
       <c r="C15" s="9">
         <v>42</v>
@@ -2774,17 +2776,17 @@
       </c>
     </row>
     <row r="16" spans="1:4">
-      <c r="A16" s="11" t="s">
+      <c r="A16" s="4" t="s">
         <v>77</v>
       </c>
-      <c r="B16" s="11">
+      <c r="B16" s="5">
         <v>1</v>
       </c>
-      <c r="C16" s="11">
-        <v>2650</v>
-      </c>
-      <c r="D16" s="11">
-        <v>2838</v>
+      <c r="C16" s="9">
+        <v>2596</v>
+      </c>
+      <c r="D16" s="9">
+        <v>2782</v>
       </c>
     </row>
     <row r="18" spans="1:4">
@@ -2810,182 +2812,182 @@
       <c r="A20" t="s">
         <v>91</v>
       </c>
-      <c r="B20" s="8">
-        <v>0.1951020408163265</v>
+      <c r="B20" s="12">
+        <v>0.1949685534591195</v>
       </c>
       <c r="C20" s="9">
-        <v>478</v>
+        <v>527</v>
       </c>
       <c r="D20" s="9">
-        <v>510</v>
+        <v>561</v>
       </c>
     </row>
     <row r="21" spans="1:4">
       <c r="A21" t="s">
         <v>93</v>
       </c>
-      <c r="B21" s="8">
-        <v>0.1346938775510204</v>
+      <c r="B21" s="12">
+        <v>0.1342952275249722</v>
       </c>
       <c r="C21" s="9">
-        <v>330</v>
+        <v>363</v>
       </c>
       <c r="D21" s="9">
-        <v>353</v>
+        <v>388</v>
       </c>
     </row>
     <row r="22" spans="1:4">
       <c r="A22" t="s">
         <v>92</v>
       </c>
-      <c r="B22" s="8">
-        <v>0.1183673469387755</v>
+      <c r="B22" s="12">
+        <v>0.1187569367369589</v>
       </c>
       <c r="C22" s="9">
-        <v>290</v>
+        <v>321</v>
       </c>
       <c r="D22" s="9">
-        <v>310</v>
+        <v>343</v>
       </c>
     </row>
     <row r="23" spans="1:4">
       <c r="A23" t="s">
         <v>99</v>
       </c>
-      <c r="B23" s="8">
-        <v>0.09918367346938775</v>
+      <c r="B23" s="12">
+        <v>0.09914909359970403</v>
       </c>
       <c r="C23" s="9">
-        <v>243</v>
+        <v>268</v>
       </c>
       <c r="D23" s="9">
-        <v>261</v>
+        <v>286</v>
       </c>
     </row>
     <row r="24" spans="1:4">
       <c r="A24" t="s">
         <v>103</v>
       </c>
-      <c r="B24" s="8">
-        <v>0.09795918367346938</v>
+      <c r="B24" s="12">
+        <v>0.09766925638179801</v>
       </c>
       <c r="C24" s="9">
-        <v>240</v>
+        <v>264</v>
       </c>
       <c r="D24" s="9">
-        <v>256</v>
+        <v>283</v>
       </c>
     </row>
     <row r="25" spans="1:4">
       <c r="A25" t="s">
         <v>95</v>
       </c>
-      <c r="B25" s="8">
-        <v>0.09346938775510204</v>
+      <c r="B25" s="12">
+        <v>0.09322974472807991</v>
       </c>
       <c r="C25" s="9">
-        <v>229</v>
+        <v>252</v>
       </c>
       <c r="D25" s="9">
-        <v>245</v>
+        <v>269</v>
       </c>
     </row>
     <row r="26" spans="1:4">
       <c r="A26" t="s">
         <v>97</v>
       </c>
-      <c r="B26" s="8">
-        <v>0.06163265306122449</v>
+      <c r="B26" s="12">
+        <v>0.06215316315205328</v>
       </c>
       <c r="C26" s="9">
-        <v>151</v>
+        <v>168</v>
       </c>
       <c r="D26" s="9">
-        <v>162</v>
+        <v>180</v>
       </c>
     </row>
     <row r="27" spans="1:4">
       <c r="A27" t="s">
         <v>98</v>
       </c>
-      <c r="B27" s="8">
-        <v>0.05591836734693877</v>
+      <c r="B27" s="12">
+        <v>0.05623381428042915</v>
       </c>
       <c r="C27" s="9">
-        <v>137</v>
+        <v>152</v>
       </c>
       <c r="D27" s="9">
-        <v>148</v>
+        <v>163</v>
       </c>
     </row>
     <row r="28" spans="1:4">
       <c r="A28" t="s">
         <v>96</v>
       </c>
-      <c r="B28" s="8">
-        <v>0.05061224489795919</v>
+      <c r="B28" s="12">
+        <v>0.04994450610432852</v>
       </c>
       <c r="C28" s="9">
-        <v>124</v>
+        <v>135</v>
       </c>
       <c r="D28" s="9">
-        <v>135</v>
+        <v>146</v>
       </c>
     </row>
     <row r="29" spans="1:4">
       <c r="A29" t="s">
         <v>104</v>
       </c>
-      <c r="B29" s="8">
-        <v>0.04816326530612245</v>
+      <c r="B29" s="12">
+        <v>0.04809470958194598</v>
       </c>
       <c r="C29" s="9">
-        <v>118</v>
+        <v>130</v>
       </c>
       <c r="D29" s="9">
-        <v>127</v>
+        <v>140</v>
       </c>
     </row>
     <row r="30" spans="1:4">
       <c r="A30" t="s">
         <v>105</v>
       </c>
-      <c r="B30" s="8">
-        <v>0.02448979591836735</v>
+      <c r="B30" s="12">
+        <v>0.0244173140954495</v>
       </c>
       <c r="C30" s="9">
-        <v>60</v>
+        <v>66</v>
       </c>
       <c r="D30" s="9">
-        <v>66</v>
+        <v>72</v>
       </c>
     </row>
     <row r="31" spans="1:4">
       <c r="A31" t="s">
         <v>101</v>
       </c>
-      <c r="B31" s="8">
-        <v>0.02040816326530612</v>
+      <c r="B31" s="12">
+        <v>0.02108768035516093</v>
       </c>
       <c r="C31" s="9">
-        <v>50</v>
+        <v>57</v>
       </c>
       <c r="D31" s="9">
-        <v>55</v>
+        <v>62</v>
       </c>
     </row>
     <row r="32" spans="1:4">
-      <c r="A32" s="11" t="s">
+      <c r="A32" s="4" t="s">
         <v>77</v>
       </c>
-      <c r="B32" s="11">
+      <c r="B32" s="5">
         <v>1</v>
       </c>
-      <c r="C32" s="11">
-        <v>2450</v>
-      </c>
-      <c r="D32" s="11">
-        <v>2628</v>
+      <c r="C32" s="9">
+        <v>2703</v>
+      </c>
+      <c r="D32" s="9">
+        <v>2893</v>
       </c>
     </row>
     <row r="34" spans="1:4">
@@ -3011,182 +3013,182 @@
       <c r="A36" t="s">
         <v>93</v>
       </c>
-      <c r="B36" s="8">
-        <v>0.1227118644067797</v>
+      <c r="B36" s="12">
+        <v>0.1228644129407488</v>
       </c>
       <c r="C36" s="9">
-        <v>362</v>
+        <v>338</v>
       </c>
       <c r="D36" s="9">
-        <v>386</v>
+        <v>361</v>
       </c>
     </row>
     <row r="37" spans="1:4">
       <c r="A37" t="s">
         <v>95</v>
       </c>
-      <c r="B37" s="8">
-        <v>0.1196610169491525</v>
+      <c r="B37" s="12">
+        <v>0.1195928753180662</v>
       </c>
       <c r="C37" s="9">
-        <v>353</v>
+        <v>329</v>
       </c>
       <c r="D37" s="9">
-        <v>376</v>
+        <v>351</v>
       </c>
     </row>
     <row r="38" spans="1:4">
       <c r="A38" t="s">
         <v>91</v>
       </c>
-      <c r="B38" s="8">
-        <v>0.1074576271186441</v>
+      <c r="B38" s="12">
+        <v>0.1075972373682297</v>
       </c>
       <c r="C38" s="9">
+        <v>296</v>
+      </c>
+      <c r="D38" s="9">
         <v>317</v>
-      </c>
-      <c r="D38" s="9">
-        <v>340</v>
       </c>
     </row>
     <row r="39" spans="1:4">
       <c r="A39" t="s">
         <v>103</v>
       </c>
-      <c r="B39" s="8">
-        <v>0.09966101694915254</v>
+      <c r="B39" s="12">
+        <v>0.0999636495819702</v>
       </c>
       <c r="C39" s="9">
+        <v>275</v>
+      </c>
+      <c r="D39" s="9">
         <v>294</v>
-      </c>
-      <c r="D39" s="9">
-        <v>315</v>
       </c>
     </row>
     <row r="40" spans="1:4">
       <c r="A40" t="s">
         <v>94</v>
       </c>
-      <c r="B40" s="8">
-        <v>0.09593220338983051</v>
+      <c r="B40" s="12">
+        <v>0.09632860777898945</v>
       </c>
       <c r="C40" s="9">
-        <v>283</v>
+        <v>265</v>
       </c>
       <c r="D40" s="9">
-        <v>302</v>
+        <v>284</v>
       </c>
     </row>
     <row r="41" spans="1:4">
       <c r="A41" t="s">
         <v>97</v>
       </c>
-      <c r="B41" s="8">
-        <v>0.08915254237288135</v>
+      <c r="B41" s="12">
+        <v>0.08869501999272991</v>
       </c>
       <c r="C41" s="9">
-        <v>263</v>
+        <v>244</v>
       </c>
       <c r="D41" s="9">
-        <v>282</v>
+        <v>260</v>
       </c>
     </row>
     <row r="42" spans="1:4">
       <c r="A42" t="s">
         <v>92</v>
       </c>
-      <c r="B42" s="8">
-        <v>0.07559322033898305</v>
+      <c r="B42" s="12">
+        <v>0.07560886950199927</v>
       </c>
       <c r="C42" s="9">
-        <v>223</v>
+        <v>208</v>
       </c>
       <c r="D42" s="9">
-        <v>240</v>
+        <v>224</v>
       </c>
     </row>
     <row r="43" spans="1:4">
       <c r="A43" t="s">
         <v>104</v>
       </c>
-      <c r="B43" s="8">
-        <v>0.07220338983050847</v>
+      <c r="B43" s="12">
+        <v>0.07161032351872046</v>
       </c>
       <c r="C43" s="9">
-        <v>213</v>
+        <v>197</v>
       </c>
       <c r="D43" s="9">
-        <v>229</v>
+        <v>212</v>
       </c>
     </row>
     <row r="44" spans="1:4">
       <c r="A44" t="s">
         <v>99</v>
       </c>
-      <c r="B44" s="8">
-        <v>0.07220338983050847</v>
+      <c r="B44" s="12">
+        <v>0.07233733187931661</v>
       </c>
       <c r="C44" s="9">
-        <v>213</v>
+        <v>199</v>
       </c>
       <c r="D44" s="9">
-        <v>230</v>
+        <v>215</v>
       </c>
     </row>
     <row r="45" spans="1:4">
       <c r="A45" t="s">
         <v>96</v>
       </c>
-      <c r="B45" s="8">
-        <v>0.05389830508474576</v>
+      <c r="B45" s="12">
+        <v>0.05452562704471101</v>
       </c>
       <c r="C45" s="9">
-        <v>159</v>
+        <v>150</v>
       </c>
       <c r="D45" s="9">
-        <v>172</v>
+        <v>162</v>
       </c>
     </row>
     <row r="46" spans="1:4">
       <c r="A46" t="s">
         <v>105</v>
       </c>
-      <c r="B46" s="8">
-        <v>0.04779661016949153</v>
+      <c r="B46" s="12">
+        <v>0.04725554343874955</v>
       </c>
       <c r="C46" s="9">
-        <v>141</v>
+        <v>130</v>
       </c>
       <c r="D46" s="9">
-        <v>153</v>
+        <v>142</v>
       </c>
     </row>
     <row r="47" spans="1:4">
       <c r="A47" t="s">
         <v>101</v>
       </c>
-      <c r="B47" s="8">
-        <v>0.04372881355932203</v>
+      <c r="B47" s="12">
+        <v>0.04362050163576881</v>
       </c>
       <c r="C47" s="9">
-        <v>129</v>
+        <v>120</v>
       </c>
       <c r="D47" s="9">
-        <v>140</v>
+        <v>130</v>
       </c>
     </row>
     <row r="48" spans="1:4">
-      <c r="A48" s="11" t="s">
+      <c r="A48" s="4" t="s">
         <v>77</v>
       </c>
-      <c r="B48" s="11">
+      <c r="B48" s="5">
         <v>1</v>
       </c>
-      <c r="C48" s="11">
-        <v>2950</v>
-      </c>
-      <c r="D48" s="11">
-        <v>3165</v>
+      <c r="C48" s="9">
+        <v>2751</v>
+      </c>
+      <c r="D48" s="9">
+        <v>2952</v>
       </c>
     </row>
   </sheetData>
@@ -3237,22 +3239,22 @@
         <v>111</v>
       </c>
       <c r="B5">
+        <v>89</v>
+      </c>
+      <c r="C5">
+        <v>148</v>
+      </c>
+      <c r="D5">
+        <v>170</v>
+      </c>
+      <c r="E5">
         <v>90</v>
       </c>
-      <c r="C5">
-        <v>151</v>
-      </c>
-      <c r="D5">
-        <v>174</v>
-      </c>
-      <c r="E5">
-        <v>91</v>
-      </c>
       <c r="F5">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="G5">
-        <v>533</v>
+        <v>523</v>
       </c>
     </row>
     <row r="6" spans="1:7">
@@ -3260,22 +3262,22 @@
         <v>112</v>
       </c>
       <c r="B6">
+        <v>95</v>
+      </c>
+      <c r="C6">
+        <v>157</v>
+      </c>
+      <c r="D6">
+        <v>181</v>
+      </c>
+      <c r="E6">
         <v>96</v>
       </c>
-      <c r="C6">
-        <v>161</v>
-      </c>
-      <c r="D6">
-        <v>185</v>
-      </c>
-      <c r="E6">
-        <v>97</v>
-      </c>
       <c r="F6">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="G6">
-        <v>568</v>
+        <v>557</v>
       </c>
     </row>
     <row r="7" spans="1:7">
@@ -3283,22 +3285,22 @@
         <v>113</v>
       </c>
       <c r="B7">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C7">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="D7">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="E7">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="F7">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="G7">
-        <v>340</v>
+        <v>332</v>
       </c>
     </row>
     <row r="8" spans="1:7">
@@ -3306,22 +3308,22 @@
         <v>114</v>
       </c>
       <c r="B8">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="C8">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="D8">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="E8">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="F8">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="G8">
-        <v>364</v>
+        <v>356</v>
       </c>
     </row>
     <row r="9" spans="1:7">
@@ -3329,22 +3331,22 @@
         <v>115</v>
       </c>
       <c r="B9">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C9">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="D9">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="E9">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="F9">
         <v>21</v>
       </c>
       <c r="G9">
-        <v>320</v>
+        <v>314</v>
       </c>
     </row>
     <row r="10" spans="1:7">
@@ -3352,22 +3354,22 @@
         <v>116</v>
       </c>
       <c r="B10">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="C10">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="D10">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="E10">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="F10">
         <v>23</v>
       </c>
       <c r="G10">
-        <v>342</v>
+        <v>336</v>
       </c>
     </row>
     <row r="11" spans="1:7">
@@ -3375,22 +3377,22 @@
         <v>117</v>
       </c>
       <c r="B11">
+        <v>54</v>
+      </c>
+      <c r="C11">
         <v>56</v>
       </c>
-      <c r="C11">
+      <c r="D11">
+        <v>62</v>
+      </c>
+      <c r="E11">
         <v>57</v>
       </c>
-      <c r="D11">
-        <v>64</v>
-      </c>
-      <c r="E11">
-        <v>58</v>
-      </c>
       <c r="F11">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="G11">
-        <v>266</v>
+        <v>259</v>
       </c>
     </row>
     <row r="12" spans="1:7">
@@ -3398,22 +3400,22 @@
         <v>118</v>
       </c>
       <c r="B12">
+        <v>58</v>
+      </c>
+      <c r="C12">
         <v>60</v>
       </c>
-      <c r="C12">
+      <c r="D12">
+        <v>66</v>
+      </c>
+      <c r="E12">
         <v>61</v>
       </c>
-      <c r="D12">
-        <v>68</v>
-      </c>
-      <c r="E12">
-        <v>62</v>
-      </c>
       <c r="F12">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="G12">
-        <v>284</v>
+        <v>277</v>
       </c>
     </row>
     <row r="13" spans="1:7">
@@ -3421,22 +3423,22 @@
         <v>119</v>
       </c>
       <c r="B13">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C13">
+        <v>57</v>
+      </c>
+      <c r="D13">
+        <v>78</v>
+      </c>
+      <c r="E13">
         <v>58</v>
       </c>
-      <c r="D13">
-        <v>80</v>
-      </c>
-      <c r="E13">
-        <v>59</v>
-      </c>
       <c r="F13">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="G13">
-        <v>255</v>
+        <v>249</v>
       </c>
     </row>
     <row r="14" spans="1:7">
@@ -3444,22 +3446,22 @@
         <v>120</v>
       </c>
       <c r="B14">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C14">
+        <v>61</v>
+      </c>
+      <c r="D14">
+        <v>83</v>
+      </c>
+      <c r="E14">
         <v>62</v>
       </c>
-      <c r="D14">
-        <v>85</v>
-      </c>
-      <c r="E14">
-        <v>63</v>
-      </c>
       <c r="F14">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="G14">
-        <v>273</v>
+        <v>267</v>
       </c>
     </row>
     <row r="15" spans="1:7">
@@ -3467,22 +3469,22 @@
         <v>121</v>
       </c>
       <c r="B15">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C15">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D15">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="E15">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="F15">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="G15">
-        <v>233</v>
+        <v>228</v>
       </c>
     </row>
     <row r="16" spans="1:7">
@@ -3490,22 +3492,22 @@
         <v>122</v>
       </c>
       <c r="B16">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C16">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="D16">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="E16">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="F16">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="G16">
-        <v>250</v>
+        <v>245</v>
       </c>
     </row>
     <row r="17" spans="1:7">
@@ -3516,10 +3518,10 @@
         <v>31</v>
       </c>
       <c r="C17">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="D17">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="E17">
         <v>31</v>
@@ -3528,7 +3530,7 @@
         <v>17</v>
       </c>
       <c r="G17">
-        <v>216</v>
+        <v>212</v>
       </c>
     </row>
     <row r="18" spans="1:7">
@@ -3539,10 +3541,10 @@
         <v>33</v>
       </c>
       <c r="C18">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="D18">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="E18">
         <v>33</v>
@@ -3551,7 +3553,7 @@
         <v>19</v>
       </c>
       <c r="G18">
-        <v>231</v>
+        <v>227</v>
       </c>
     </row>
     <row r="19" spans="1:7">
@@ -3559,22 +3561,22 @@
         <v>125</v>
       </c>
       <c r="B19">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C19">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="D19">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="E19">
         <v>23</v>
       </c>
       <c r="F19">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="G19">
-        <v>174</v>
+        <v>170</v>
       </c>
     </row>
     <row r="20" spans="1:7">
@@ -3582,22 +3584,22 @@
         <v>126</v>
       </c>
       <c r="B20">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C20">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="D20">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="E20">
         <v>25</v>
       </c>
       <c r="F20">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G20">
-        <v>187</v>
+        <v>183</v>
       </c>
     </row>
     <row r="21" spans="1:7">
@@ -3608,19 +3610,19 @@
         <v>22</v>
       </c>
       <c r="C21">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="D21">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="E21">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="F21">
         <v>10</v>
       </c>
       <c r="G21">
-        <v>146</v>
+        <v>143</v>
       </c>
     </row>
     <row r="22" spans="1:7">
@@ -3631,19 +3633,19 @@
         <v>24</v>
       </c>
       <c r="C22">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="D22">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="E22">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="F22">
         <v>11</v>
       </c>
       <c r="G22">
-        <v>158</v>
+        <v>154</v>
       </c>
     </row>
     <row r="23" spans="1:7">
@@ -3654,7 +3656,7 @@
         <v>22</v>
       </c>
       <c r="C23">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="D23">
         <v>32</v>
@@ -3666,7 +3668,7 @@
         <v>11</v>
       </c>
       <c r="G23">
-        <v>125</v>
+        <v>124</v>
       </c>
     </row>
     <row r="24" spans="1:7">
@@ -3677,7 +3679,7 @@
         <v>24</v>
       </c>
       <c r="C24">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="D24">
         <v>34</v>
@@ -3689,7 +3691,7 @@
         <v>12</v>
       </c>
       <c r="G24">
-        <v>134</v>
+        <v>133</v>
       </c>
     </row>
     <row r="25" spans="1:7">
@@ -3771,22 +3773,22 @@
         <v>111</v>
       </c>
       <c r="B30">
-        <v>118</v>
+        <v>130</v>
       </c>
       <c r="C30">
-        <v>143</v>
+        <v>158</v>
       </c>
       <c r="D30">
-        <v>119</v>
+        <v>131</v>
       </c>
       <c r="E30">
-        <v>62</v>
+        <v>68</v>
       </c>
       <c r="F30">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="G30">
-        <v>478</v>
+        <v>527</v>
       </c>
     </row>
     <row r="31" spans="1:7">
@@ -3794,22 +3796,22 @@
         <v>112</v>
       </c>
       <c r="B31">
-        <v>126</v>
+        <v>138</v>
       </c>
       <c r="C31">
-        <v>152</v>
+        <v>168</v>
       </c>
       <c r="D31">
-        <v>127</v>
+        <v>139</v>
       </c>
       <c r="E31">
-        <v>66</v>
+        <v>73</v>
       </c>
       <c r="F31">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="G31">
-        <v>510</v>
+        <v>561</v>
       </c>
     </row>
     <row r="32" spans="1:7">
@@ -3817,22 +3819,22 @@
         <v>115</v>
       </c>
       <c r="B32">
-        <v>68</v>
+        <v>75</v>
       </c>
       <c r="C32">
-        <v>106</v>
+        <v>117</v>
       </c>
       <c r="D32">
-        <v>83</v>
+        <v>91</v>
       </c>
       <c r="E32">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="F32">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="G32">
-        <v>330</v>
+        <v>363</v>
       </c>
     </row>
     <row r="33" spans="1:7">
@@ -3840,22 +3842,22 @@
         <v>116</v>
       </c>
       <c r="B33">
-        <v>73</v>
+        <v>80</v>
       </c>
       <c r="C33">
-        <v>113</v>
+        <v>125</v>
       </c>
       <c r="D33">
-        <v>88</v>
+        <v>97</v>
       </c>
       <c r="E33">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="F33">
-        <v>42</v>
+        <v>46</v>
       </c>
       <c r="G33">
-        <v>353</v>
+        <v>388</v>
       </c>
     </row>
     <row r="34" spans="1:7">
@@ -3863,22 +3865,22 @@
         <v>113</v>
       </c>
       <c r="B34">
-        <v>41</v>
+        <v>45</v>
       </c>
       <c r="C34">
+        <v>88</v>
+      </c>
+      <c r="D34">
         <v>79</v>
       </c>
-      <c r="D34">
-        <v>71</v>
-      </c>
       <c r="E34">
-        <v>67</v>
+        <v>74</v>
       </c>
       <c r="F34">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="G34">
-        <v>290</v>
+        <v>321</v>
       </c>
     </row>
     <row r="35" spans="1:7">
@@ -3886,22 +3888,22 @@
         <v>114</v>
       </c>
       <c r="B35">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="C35">
+        <v>94</v>
+      </c>
+      <c r="D35">
         <v>84</v>
       </c>
-      <c r="D35">
-        <v>76</v>
-      </c>
       <c r="E35">
-        <v>72</v>
+        <v>79</v>
       </c>
       <c r="F35">
-        <v>34</v>
+        <v>38</v>
       </c>
       <c r="G35">
-        <v>310</v>
+        <v>343</v>
       </c>
     </row>
     <row r="36" spans="1:7">
@@ -3909,22 +3911,22 @@
         <v>127</v>
       </c>
       <c r="B36">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="C36">
-        <v>67</v>
+        <v>74</v>
       </c>
       <c r="D36">
-        <v>59</v>
+        <v>65</v>
       </c>
       <c r="E36">
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="F36">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="G36">
-        <v>243</v>
+        <v>268</v>
       </c>
     </row>
     <row r="37" spans="1:7">
@@ -3932,22 +3934,22 @@
         <v>128</v>
       </c>
       <c r="B37">
-        <v>55</v>
+        <v>60</v>
       </c>
       <c r="C37">
-        <v>72</v>
+        <v>79</v>
       </c>
       <c r="D37">
-        <v>63</v>
+        <v>69</v>
       </c>
       <c r="E37">
-        <v>41</v>
+        <v>45</v>
       </c>
       <c r="F37">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="G37">
-        <v>261</v>
+        <v>286</v>
       </c>
     </row>
     <row r="38" spans="1:7">
@@ -3955,22 +3957,22 @@
         <v>134</v>
       </c>
       <c r="B38">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="C38">
-        <v>65</v>
+        <v>72</v>
       </c>
       <c r="D38">
-        <v>76</v>
+        <v>84</v>
       </c>
       <c r="E38">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="F38">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="G38">
-        <v>240</v>
+        <v>264</v>
       </c>
     </row>
     <row r="39" spans="1:7">
@@ -3978,22 +3980,22 @@
         <v>135</v>
       </c>
       <c r="B39">
-        <v>52</v>
+        <v>57</v>
       </c>
       <c r="C39">
-        <v>69</v>
+        <v>77</v>
       </c>
       <c r="D39">
-        <v>81</v>
+        <v>90</v>
       </c>
       <c r="E39">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="F39">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="G39">
-        <v>256</v>
+        <v>283</v>
       </c>
     </row>
     <row r="40" spans="1:7">
@@ -4001,22 +4003,22 @@
         <v>119</v>
       </c>
       <c r="B40">
-        <v>43</v>
+        <v>48</v>
       </c>
       <c r="C40">
-        <v>72</v>
+        <v>80</v>
       </c>
       <c r="D40">
-        <v>56</v>
+        <v>61</v>
       </c>
       <c r="E40">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="F40">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="G40">
-        <v>229</v>
+        <v>252</v>
       </c>
     </row>
     <row r="41" spans="1:7">
@@ -4024,22 +4026,22 @@
         <v>120</v>
       </c>
       <c r="B41">
-        <v>46</v>
+        <v>51</v>
       </c>
       <c r="C41">
-        <v>77</v>
+        <v>85</v>
       </c>
       <c r="D41">
-        <v>60</v>
+        <v>65</v>
       </c>
       <c r="E41">
-        <v>34</v>
+        <v>38</v>
       </c>
       <c r="F41">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="G41">
-        <v>245</v>
+        <v>269</v>
       </c>
     </row>
     <row r="42" spans="1:7">
@@ -4047,22 +4049,22 @@
         <v>123</v>
       </c>
       <c r="B42">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="C42">
-        <v>47</v>
+        <v>52</v>
       </c>
       <c r="D42">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="E42">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="F42">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="G42">
-        <v>151</v>
+        <v>168</v>
       </c>
     </row>
     <row r="43" spans="1:7">
@@ -4070,22 +4072,22 @@
         <v>124</v>
       </c>
       <c r="B43">
-        <v>40</v>
+        <v>44</v>
       </c>
       <c r="C43">
-        <v>50</v>
+        <v>56</v>
       </c>
       <c r="D43">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="E43">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="F43">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="G43">
-        <v>162</v>
+        <v>180</v>
       </c>
     </row>
     <row r="44" spans="1:7">
@@ -4093,22 +4095,22 @@
         <v>125</v>
       </c>
       <c r="B44">
-        <v>43</v>
+        <v>48</v>
       </c>
       <c r="C44">
-        <v>41</v>
+        <v>45</v>
       </c>
       <c r="D44">
-        <v>34</v>
+        <v>38</v>
       </c>
       <c r="E44">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="F44">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="G44">
-        <v>137</v>
+        <v>152</v>
       </c>
     </row>
     <row r="45" spans="1:7">
@@ -4116,22 +4118,22 @@
         <v>126</v>
       </c>
       <c r="B45">
-        <v>46</v>
+        <v>51</v>
       </c>
       <c r="C45">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="D45">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="E45">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F45">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="G45">
-        <v>148</v>
+        <v>163</v>
       </c>
     </row>
     <row r="46" spans="1:7">
@@ -4139,22 +4141,22 @@
         <v>121</v>
       </c>
       <c r="B46">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C46">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="D46">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="E46">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="F46">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="G46">
-        <v>124</v>
+        <v>135</v>
       </c>
     </row>
     <row r="47" spans="1:7">
@@ -4162,22 +4164,22 @@
         <v>122</v>
       </c>
       <c r="B47">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C47">
-        <v>42</v>
+        <v>46</v>
       </c>
       <c r="D47">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="E47">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="F47">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="G47">
-        <v>135</v>
+        <v>146</v>
       </c>
     </row>
     <row r="48" spans="1:7">
@@ -4185,22 +4187,22 @@
         <v>136</v>
       </c>
       <c r="B48">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="C48">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="D48">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="E48">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="F48">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="G48">
-        <v>118</v>
+        <v>130</v>
       </c>
     </row>
     <row r="49" spans="1:9">
@@ -4208,22 +4210,22 @@
         <v>137</v>
       </c>
       <c r="B49">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="C49">
-        <v>33</v>
+        <v>37</v>
       </c>
       <c r="D49">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="E49">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="F49">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="G49">
-        <v>127</v>
+        <v>140</v>
       </c>
     </row>
     <row r="50" spans="1:9">
@@ -4231,22 +4233,22 @@
         <v>138</v>
       </c>
       <c r="B50">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C50">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D50">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E50">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="F50">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="G50">
-        <v>60</v>
+        <v>66</v>
       </c>
     </row>
     <row r="51" spans="1:9">
@@ -4254,22 +4256,22 @@
         <v>139</v>
       </c>
       <c r="B51">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C51">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D51">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E51">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="F51">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="G51">
-        <v>66</v>
+        <v>72</v>
       </c>
     </row>
     <row r="52" spans="1:9">
@@ -4277,22 +4279,22 @@
         <v>131</v>
       </c>
       <c r="B52">
+        <v>16</v>
+      </c>
+      <c r="C52">
         <v>14</v>
       </c>
-      <c r="C52">
+      <c r="D52">
         <v>12</v>
       </c>
-      <c r="D52">
-        <v>11</v>
-      </c>
       <c r="E52">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F52">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="G52">
-        <v>50</v>
+        <v>57</v>
       </c>
     </row>
     <row r="53" spans="1:9">
@@ -4300,22 +4302,22 @@
         <v>132</v>
       </c>
       <c r="B53">
+        <v>17</v>
+      </c>
+      <c r="C53">
         <v>15</v>
       </c>
-      <c r="C53">
+      <c r="D53">
         <v>13</v>
       </c>
-      <c r="D53">
-        <v>12</v>
-      </c>
       <c r="E53">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="F53">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="G53">
-        <v>55</v>
+        <v>62</v>
       </c>
     </row>
     <row r="55" spans="1:9">
@@ -4357,28 +4359,28 @@
         <v>115</v>
       </c>
       <c r="B57">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="C57">
-        <v>66</v>
+        <v>61</v>
       </c>
       <c r="D57">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="E57">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="F57">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="G57">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="H57">
-        <v>61</v>
+        <v>56</v>
       </c>
       <c r="I57">
-        <v>362</v>
+        <v>338</v>
       </c>
     </row>
     <row r="58" spans="1:9">
@@ -4386,28 +4388,28 @@
         <v>116</v>
       </c>
       <c r="B58">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="C58">
-        <v>70</v>
+        <v>65</v>
       </c>
       <c r="D58">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="E58">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="F58">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="G58">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="H58">
-        <v>65</v>
+        <v>60</v>
       </c>
       <c r="I58">
-        <v>386</v>
+        <v>361</v>
       </c>
     </row>
     <row r="59" spans="1:9">
@@ -4415,28 +4417,28 @@
         <v>119</v>
       </c>
       <c r="B59">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="C59">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="D59">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="E59">
-        <v>61</v>
+        <v>56</v>
       </c>
       <c r="F59">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="G59">
-        <v>68</v>
+        <v>63</v>
       </c>
       <c r="H59">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="I59">
-        <v>353</v>
+        <v>329</v>
       </c>
     </row>
     <row r="60" spans="1:9">
@@ -4444,28 +4446,28 @@
         <v>120</v>
       </c>
       <c r="B60">
-        <v>68</v>
+        <v>64</v>
       </c>
       <c r="C60">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="D60">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="E60">
-        <v>65</v>
+        <v>60</v>
       </c>
       <c r="F60">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="G60">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="H60">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="I60">
-        <v>376</v>
+        <v>351</v>
       </c>
     </row>
     <row r="61" spans="1:9">
@@ -4473,28 +4475,28 @@
         <v>111</v>
       </c>
       <c r="B61">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="C61">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="D61">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="E61">
-        <v>53</v>
+        <v>49</v>
       </c>
       <c r="F61">
-        <v>53</v>
+        <v>49</v>
       </c>
       <c r="G61">
-        <v>59</v>
+        <v>55</v>
       </c>
       <c r="H61">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="I61">
-        <v>317</v>
+        <v>296</v>
       </c>
     </row>
     <row r="62" spans="1:9">
@@ -4502,28 +4504,28 @@
         <v>112</v>
       </c>
       <c r="B62">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C62">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="D62">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="E62">
-        <v>57</v>
+        <v>52</v>
       </c>
       <c r="F62">
-        <v>57</v>
+        <v>52</v>
       </c>
       <c r="G62">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="H62">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="I62">
-        <v>340</v>
+        <v>317</v>
       </c>
     </row>
     <row r="63" spans="1:9">
@@ -4531,28 +4533,28 @@
         <v>134</v>
       </c>
       <c r="B63">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="C63">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="D63">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="E63">
-        <v>52</v>
+        <v>48</v>
       </c>
       <c r="F63">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="G63">
+        <v>38</v>
+      </c>
+      <c r="H63">
         <v>40</v>
       </c>
-      <c r="H63">
-        <v>43</v>
-      </c>
       <c r="I63">
-        <v>294</v>
+        <v>275</v>
       </c>
     </row>
     <row r="64" spans="1:9">
@@ -4560,28 +4562,28 @@
         <v>135</v>
       </c>
       <c r="B64">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="C64">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="D64">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="E64">
-        <v>56</v>
+        <v>51</v>
       </c>
       <c r="F64">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="G64">
+        <v>41</v>
+      </c>
+      <c r="H64">
         <v>43</v>
       </c>
-      <c r="H64">
-        <v>46</v>
-      </c>
       <c r="I64">
-        <v>315</v>
+        <v>294</v>
       </c>
     </row>
     <row r="65" spans="1:9">
@@ -4589,28 +4591,28 @@
         <v>117</v>
       </c>
       <c r="B65">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="C65">
+        <v>38</v>
+      </c>
+      <c r="D65">
+        <v>41</v>
+      </c>
+      <c r="E65">
         <v>40</v>
       </c>
-      <c r="D65">
-        <v>44</v>
-      </c>
-      <c r="E65">
+      <c r="F65">
         <v>43</v>
       </c>
-      <c r="F65">
+      <c r="G65">
         <v>47</v>
       </c>
-      <c r="G65">
-        <v>50</v>
-      </c>
       <c r="H65">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="I65">
-        <v>283</v>
+        <v>265</v>
       </c>
     </row>
     <row r="66" spans="1:9">
@@ -4618,28 +4620,28 @@
         <v>118</v>
       </c>
       <c r="B66">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="C66">
+        <v>41</v>
+      </c>
+      <c r="D66">
+        <v>44</v>
+      </c>
+      <c r="E66">
         <v>43</v>
       </c>
-      <c r="D66">
-        <v>47</v>
-      </c>
-      <c r="E66">
+      <c r="F66">
         <v>46</v>
       </c>
-      <c r="F66">
+      <c r="G66">
         <v>50</v>
       </c>
-      <c r="G66">
-        <v>53</v>
-      </c>
       <c r="H66">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="I66">
-        <v>302</v>
+        <v>284</v>
       </c>
     </row>
     <row r="67" spans="1:9">
@@ -4647,28 +4649,28 @@
         <v>123</v>
       </c>
       <c r="B67">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="C67">
-        <v>52</v>
+        <v>48</v>
       </c>
       <c r="D67">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="E67">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="F67">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="G67">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="H67">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="I67">
-        <v>263</v>
+        <v>244</v>
       </c>
     </row>
     <row r="68" spans="1:9">
@@ -4676,28 +4678,28 @@
         <v>124</v>
       </c>
       <c r="B68">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="C68">
-        <v>56</v>
+        <v>51</v>
       </c>
       <c r="D68">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="E68">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="F68">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="G68">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="H68">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="I68">
-        <v>282</v>
+        <v>260</v>
       </c>
     </row>
     <row r="69" spans="1:9">
@@ -4705,28 +4707,28 @@
         <v>113</v>
       </c>
       <c r="B69">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="C69">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="D69">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="E69">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F69">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G69">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="H69">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="I69">
-        <v>223</v>
+        <v>208</v>
       </c>
     </row>
     <row r="70" spans="1:9">
@@ -4734,28 +4736,28 @@
         <v>114</v>
       </c>
       <c r="B70">
-        <v>62</v>
+        <v>58</v>
       </c>
       <c r="C70">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="D70">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="E70">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="F70">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="G70">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="H70">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="I70">
-        <v>240</v>
+        <v>224</v>
       </c>
     </row>
     <row r="71" spans="1:9">
@@ -4763,28 +4765,28 @@
         <v>136</v>
       </c>
       <c r="B71">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="C71">
-        <v>61</v>
+        <v>56</v>
       </c>
       <c r="D71">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="E71">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="F71">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="G71">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="H71">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="I71">
-        <v>213</v>
+        <v>197</v>
       </c>
     </row>
     <row r="72" spans="1:9">
@@ -4792,28 +4794,28 @@
         <v>137</v>
       </c>
       <c r="B72">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="C72">
-        <v>65</v>
+        <v>60</v>
       </c>
       <c r="D72">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="E72">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="F72">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G72">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="H72">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="I72">
-        <v>229</v>
+        <v>212</v>
       </c>
     </row>
     <row r="73" spans="1:9">
@@ -4821,28 +4823,28 @@
         <v>127</v>
       </c>
       <c r="B73">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="C73">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="D73">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="E73">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="F73">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="G73">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="H73">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="I73">
-        <v>213</v>
+        <v>199</v>
       </c>
     </row>
     <row r="74" spans="1:9">
@@ -4850,28 +4852,28 @@
         <v>128</v>
       </c>
       <c r="B74">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="C74">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="D74">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="E74">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="F74">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="G74">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="H74">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="I74">
-        <v>230</v>
+        <v>215</v>
       </c>
     </row>
     <row r="75" spans="1:9">
@@ -4879,28 +4881,28 @@
         <v>121</v>
       </c>
       <c r="B75">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="C75">
+        <v>7</v>
+      </c>
+      <c r="D75">
         <v>8</v>
       </c>
-      <c r="D75">
-        <v>9</v>
-      </c>
       <c r="E75">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="F75">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="G75">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="H75">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="I75">
-        <v>159</v>
+        <v>150</v>
       </c>
     </row>
     <row r="76" spans="1:9">
@@ -4908,28 +4910,28 @@
         <v>122</v>
       </c>
       <c r="B76">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="C76">
+        <v>8</v>
+      </c>
+      <c r="D76">
         <v>9</v>
       </c>
-      <c r="D76">
-        <v>10</v>
-      </c>
       <c r="E76">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="F76">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="G76">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="H76">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="I76">
-        <v>172</v>
+        <v>162</v>
       </c>
     </row>
     <row r="77" spans="1:9">
@@ -4937,28 +4939,28 @@
         <v>138</v>
       </c>
       <c r="B77">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="C77">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="D77">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E77">
         <v>6</v>
       </c>
       <c r="F77">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="G77">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="H77">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="I77">
-        <v>141</v>
+        <v>130</v>
       </c>
     </row>
     <row r="78" spans="1:9">
@@ -4966,28 +4968,28 @@
         <v>139</v>
       </c>
       <c r="B78">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="C78">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="D78">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="E78">
         <v>7</v>
       </c>
       <c r="F78">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G78">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="H78">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="I78">
-        <v>153</v>
+        <v>142</v>
       </c>
     </row>
     <row r="79" spans="1:9">
@@ -4995,28 +4997,28 @@
         <v>131</v>
       </c>
       <c r="B79">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C79">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D79">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E79">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="F79">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="G79">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="H79">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="I79">
-        <v>129</v>
+        <v>120</v>
       </c>
     </row>
     <row r="80" spans="1:9">
@@ -5024,28 +5026,28 @@
         <v>132</v>
       </c>
       <c r="B80">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C80">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D80">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E80">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="F80">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="G80">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="H80">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="I80">
-        <v>140</v>
+        <v>130</v>
       </c>
     </row>
   </sheetData>
@@ -5141,22 +5143,22 @@
         <v>91</v>
       </c>
       <c r="B13">
-        <v>533</v>
+        <v>523</v>
       </c>
       <c r="C13">
-        <v>568</v>
+        <v>557</v>
       </c>
       <c r="D13">
-        <v>266.5</v>
+        <v>261.5</v>
       </c>
       <c r="E13">
-        <v>284</v>
+        <v>278.5</v>
       </c>
       <c r="F13">
-        <v>319.8</v>
+        <v>313.8</v>
       </c>
       <c r="G13">
-        <v>340.8</v>
+        <v>334.2</v>
       </c>
     </row>
     <row r="14" spans="1:7">
@@ -5164,22 +5166,22 @@
         <v>92</v>
       </c>
       <c r="B14">
-        <v>340</v>
+        <v>332</v>
       </c>
       <c r="C14">
-        <v>364</v>
+        <v>356</v>
       </c>
       <c r="D14">
-        <v>170</v>
+        <v>166</v>
       </c>
       <c r="E14">
-        <v>182</v>
+        <v>178</v>
       </c>
       <c r="F14">
-        <v>204</v>
+        <v>199.2</v>
       </c>
       <c r="G14">
-        <v>218.4</v>
+        <v>213.6</v>
       </c>
     </row>
     <row r="15" spans="1:7">
@@ -5187,22 +5189,22 @@
         <v>93</v>
       </c>
       <c r="B15">
-        <v>320</v>
+        <v>314</v>
       </c>
       <c r="C15">
-        <v>342</v>
+        <v>336</v>
       </c>
       <c r="D15">
-        <v>160</v>
+        <v>157</v>
       </c>
       <c r="E15">
-        <v>171</v>
+        <v>168</v>
       </c>
       <c r="F15">
-        <v>192</v>
+        <v>188.4</v>
       </c>
       <c r="G15">
-        <v>205.2</v>
+        <v>201.6</v>
       </c>
     </row>
     <row r="16" spans="1:7">
@@ -5210,22 +5212,22 @@
         <v>94</v>
       </c>
       <c r="B16">
-        <v>266</v>
+        <v>259</v>
       </c>
       <c r="C16">
-        <v>284</v>
+        <v>277</v>
       </c>
       <c r="D16">
-        <v>133</v>
+        <v>129.5</v>
       </c>
       <c r="E16">
-        <v>142</v>
+        <v>138.5</v>
       </c>
       <c r="F16">
-        <v>159.6</v>
+        <v>155.4</v>
       </c>
       <c r="G16">
-        <v>170.4</v>
+        <v>166.2</v>
       </c>
     </row>
     <row r="17" spans="1:7">
@@ -5233,22 +5235,22 @@
         <v>95</v>
       </c>
       <c r="B17">
-        <v>255</v>
+        <v>249</v>
       </c>
       <c r="C17">
-        <v>273</v>
+        <v>267</v>
       </c>
       <c r="D17">
-        <v>127.5</v>
+        <v>124.5</v>
       </c>
       <c r="E17">
-        <v>136.5</v>
+        <v>133.5</v>
       </c>
       <c r="F17">
-        <v>153</v>
+        <v>149.4</v>
       </c>
       <c r="G17">
-        <v>163.8</v>
+        <v>160.2</v>
       </c>
     </row>
     <row r="18" spans="1:7">
@@ -5256,22 +5258,22 @@
         <v>96</v>
       </c>
       <c r="B18">
-        <v>233</v>
+        <v>228</v>
       </c>
       <c r="C18">
-        <v>250</v>
+        <v>245</v>
       </c>
       <c r="D18">
-        <v>116.5</v>
+        <v>114</v>
       </c>
       <c r="E18">
-        <v>125</v>
+        <v>122.5</v>
       </c>
       <c r="F18">
-        <v>139.8</v>
+        <v>136.8</v>
       </c>
       <c r="G18">
-        <v>150</v>
+        <v>147</v>
       </c>
     </row>
     <row r="19" spans="1:7">
@@ -5279,22 +5281,22 @@
         <v>97</v>
       </c>
       <c r="B19">
-        <v>216</v>
+        <v>212</v>
       </c>
       <c r="C19">
-        <v>231</v>
+        <v>227</v>
       </c>
       <c r="D19">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="E19">
-        <v>115.5</v>
+        <v>113.5</v>
       </c>
       <c r="F19">
-        <v>129.6</v>
+        <v>127.2</v>
       </c>
       <c r="G19">
-        <v>138.6</v>
+        <v>136.2</v>
       </c>
     </row>
     <row r="20" spans="1:7">
@@ -5302,22 +5304,22 @@
         <v>98</v>
       </c>
       <c r="B20">
-        <v>174</v>
+        <v>170</v>
       </c>
       <c r="C20">
-        <v>187</v>
+        <v>183</v>
       </c>
       <c r="D20">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="E20">
-        <v>93.5</v>
+        <v>91.5</v>
       </c>
       <c r="F20">
-        <v>104.4</v>
+        <v>102</v>
       </c>
       <c r="G20">
-        <v>112.2</v>
+        <v>109.8</v>
       </c>
     </row>
     <row r="21" spans="1:7">
@@ -5325,22 +5327,22 @@
         <v>99</v>
       </c>
       <c r="B21">
-        <v>146</v>
+        <v>143</v>
       </c>
       <c r="C21">
-        <v>158</v>
+        <v>154</v>
       </c>
       <c r="D21">
-        <v>73</v>
+        <v>71.5</v>
       </c>
       <c r="E21">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="F21">
-        <v>87.59999999999999</v>
+        <v>85.8</v>
       </c>
       <c r="G21">
-        <v>94.8</v>
+        <v>92.40000000000001</v>
       </c>
     </row>
     <row r="22" spans="1:7">
@@ -5348,22 +5350,22 @@
         <v>100</v>
       </c>
       <c r="B22">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="C22">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="D22">
-        <v>62.5</v>
+        <v>62</v>
       </c>
       <c r="E22">
-        <v>67</v>
+        <v>66.5</v>
       </c>
       <c r="F22">
-        <v>75</v>
+        <v>74.40000000000001</v>
       </c>
       <c r="G22">
-        <v>80.40000000000001</v>
+        <v>79.8</v>
       </c>
     </row>
     <row r="23" spans="1:7">
@@ -5394,22 +5396,22 @@
         <v>152</v>
       </c>
       <c r="B24" s="11">
-        <v>2650</v>
+        <v>2596</v>
       </c>
       <c r="C24" s="11">
-        <v>2838</v>
+        <v>2782</v>
       </c>
       <c r="D24" s="11">
-        <v>1325</v>
+        <v>1298</v>
       </c>
       <c r="E24" s="11">
-        <v>1419</v>
+        <v>1391</v>
       </c>
       <c r="F24" s="11">
-        <v>1590</v>
+        <v>1557.6</v>
       </c>
       <c r="G24" s="11">
-        <v>1702.8</v>
+        <v>1669.2</v>
       </c>
     </row>
     <row r="26" spans="1:7">
@@ -5445,22 +5447,22 @@
         <v>91</v>
       </c>
       <c r="B28">
-        <v>478</v>
+        <v>527</v>
       </c>
       <c r="C28">
-        <v>510</v>
+        <v>561</v>
       </c>
       <c r="D28">
-        <v>191.2</v>
+        <v>210.8</v>
       </c>
       <c r="E28">
-        <v>204</v>
+        <v>224.4</v>
       </c>
       <c r="F28">
-        <v>229.4</v>
+        <v>253</v>
       </c>
       <c r="G28">
-        <v>244.8</v>
+        <v>269.3</v>
       </c>
     </row>
     <row r="29" spans="1:7">
@@ -5468,22 +5470,22 @@
         <v>93</v>
       </c>
       <c r="B29">
-        <v>330</v>
+        <v>363</v>
       </c>
       <c r="C29">
-        <v>353</v>
+        <v>388</v>
       </c>
       <c r="D29">
-        <v>132</v>
+        <v>145.2</v>
       </c>
       <c r="E29">
-        <v>141.2</v>
+        <v>155.2</v>
       </c>
       <c r="F29">
-        <v>158.4</v>
+        <v>174.2</v>
       </c>
       <c r="G29">
-        <v>169.4</v>
+        <v>186.2</v>
       </c>
     </row>
     <row r="30" spans="1:7">
@@ -5491,22 +5493,22 @@
         <v>92</v>
       </c>
       <c r="B30">
-        <v>290</v>
+        <v>321</v>
       </c>
       <c r="C30">
-        <v>310</v>
+        <v>343</v>
       </c>
       <c r="D30">
-        <v>116</v>
+        <v>128.4</v>
       </c>
       <c r="E30">
-        <v>124</v>
+        <v>137.2</v>
       </c>
       <c r="F30">
-        <v>139.2</v>
+        <v>154.1</v>
       </c>
       <c r="G30">
-        <v>148.8</v>
+        <v>164.6</v>
       </c>
     </row>
     <row r="31" spans="1:7">
@@ -5514,22 +5516,22 @@
         <v>99</v>
       </c>
       <c r="B31">
-        <v>243</v>
+        <v>268</v>
       </c>
       <c r="C31">
-        <v>261</v>
+        <v>286</v>
       </c>
       <c r="D31">
-        <v>97.2</v>
+        <v>107.2</v>
       </c>
       <c r="E31">
-        <v>104.4</v>
+        <v>114.4</v>
       </c>
       <c r="F31">
-        <v>116.6</v>
+        <v>128.6</v>
       </c>
       <c r="G31">
-        <v>125.3</v>
+        <v>137.3</v>
       </c>
     </row>
     <row r="32" spans="1:7">
@@ -5537,22 +5539,22 @@
         <v>103</v>
       </c>
       <c r="B32">
-        <v>240</v>
+        <v>264</v>
       </c>
       <c r="C32">
-        <v>256</v>
+        <v>283</v>
       </c>
       <c r="D32">
-        <v>96</v>
+        <v>105.6</v>
       </c>
       <c r="E32">
-        <v>102.4</v>
+        <v>113.2</v>
       </c>
       <c r="F32">
-        <v>115.2</v>
+        <v>126.7</v>
       </c>
       <c r="G32">
-        <v>122.9</v>
+        <v>135.8</v>
       </c>
     </row>
     <row r="33" spans="1:7">
@@ -5560,22 +5562,22 @@
         <v>95</v>
       </c>
       <c r="B33">
-        <v>229</v>
+        <v>252</v>
       </c>
       <c r="C33">
-        <v>245</v>
+        <v>269</v>
       </c>
       <c r="D33">
-        <v>91.59999999999999</v>
+        <v>100.8</v>
       </c>
       <c r="E33">
-        <v>98</v>
+        <v>107.6</v>
       </c>
       <c r="F33">
-        <v>109.9</v>
+        <v>121</v>
       </c>
       <c r="G33">
-        <v>117.6</v>
+        <v>129.1</v>
       </c>
     </row>
     <row r="34" spans="1:7">
@@ -5583,22 +5585,22 @@
         <v>97</v>
       </c>
       <c r="B34">
-        <v>151</v>
+        <v>168</v>
       </c>
       <c r="C34">
-        <v>162</v>
+        <v>180</v>
       </c>
       <c r="D34">
-        <v>60.4</v>
+        <v>67.2</v>
       </c>
       <c r="E34">
-        <v>64.8</v>
+        <v>72</v>
       </c>
       <c r="F34">
-        <v>72.5</v>
+        <v>80.59999999999999</v>
       </c>
       <c r="G34">
-        <v>77.8</v>
+        <v>86.40000000000001</v>
       </c>
     </row>
     <row r="35" spans="1:7">
@@ -5606,22 +5608,22 @@
         <v>98</v>
       </c>
       <c r="B35">
-        <v>137</v>
+        <v>152</v>
       </c>
       <c r="C35">
-        <v>148</v>
+        <v>163</v>
       </c>
       <c r="D35">
-        <v>54.8</v>
+        <v>60.8</v>
       </c>
       <c r="E35">
-        <v>59.2</v>
+        <v>65.2</v>
       </c>
       <c r="F35">
-        <v>65.8</v>
+        <v>73</v>
       </c>
       <c r="G35">
-        <v>71</v>
+        <v>78.2</v>
       </c>
     </row>
     <row r="36" spans="1:7">
@@ -5629,22 +5631,22 @@
         <v>96</v>
       </c>
       <c r="B36">
-        <v>124</v>
+        <v>135</v>
       </c>
       <c r="C36">
-        <v>135</v>
+        <v>146</v>
       </c>
       <c r="D36">
-        <v>49.6</v>
+        <v>54</v>
       </c>
       <c r="E36">
-        <v>54</v>
+        <v>58.4</v>
       </c>
       <c r="F36">
-        <v>59.5</v>
+        <v>64.8</v>
       </c>
       <c r="G36">
-        <v>64.8</v>
+        <v>70.09999999999999</v>
       </c>
     </row>
     <row r="37" spans="1:7">
@@ -5652,22 +5654,22 @@
         <v>104</v>
       </c>
       <c r="B37">
-        <v>118</v>
+        <v>130</v>
       </c>
       <c r="C37">
-        <v>127</v>
+        <v>140</v>
       </c>
       <c r="D37">
-        <v>47.2</v>
+        <v>52</v>
       </c>
       <c r="E37">
-        <v>50.8</v>
+        <v>56</v>
       </c>
       <c r="F37">
-        <v>56.6</v>
+        <v>62.4</v>
       </c>
       <c r="G37">
-        <v>61</v>
+        <v>67.2</v>
       </c>
     </row>
     <row r="38" spans="1:7">
@@ -5675,22 +5677,22 @@
         <v>105</v>
       </c>
       <c r="B38">
-        <v>60</v>
+        <v>66</v>
       </c>
       <c r="C38">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="D38">
-        <v>24</v>
+        <v>26.4</v>
       </c>
       <c r="E38">
-        <v>26.4</v>
+        <v>28.8</v>
       </c>
       <c r="F38">
-        <v>28.8</v>
+        <v>31.7</v>
       </c>
       <c r="G38">
-        <v>31.7</v>
+        <v>34.6</v>
       </c>
     </row>
     <row r="39" spans="1:7">
@@ -5698,22 +5700,22 @@
         <v>101</v>
       </c>
       <c r="B39">
-        <v>50</v>
+        <v>57</v>
       </c>
       <c r="C39">
-        <v>55</v>
+        <v>62</v>
       </c>
       <c r="D39">
-        <v>20</v>
+        <v>22.8</v>
       </c>
       <c r="E39">
-        <v>22</v>
+        <v>24.8</v>
       </c>
       <c r="F39">
-        <v>24</v>
+        <v>27.4</v>
       </c>
       <c r="G39">
-        <v>26.4</v>
+        <v>29.8</v>
       </c>
     </row>
     <row r="40" spans="1:7">
@@ -5721,22 +5723,22 @@
         <v>154</v>
       </c>
       <c r="B40" s="11">
-        <v>2450</v>
+        <v>2703</v>
       </c>
       <c r="C40" s="11">
-        <v>2628</v>
+        <v>2893</v>
       </c>
       <c r="D40" s="11">
-        <v>980</v>
+        <v>1081.2</v>
       </c>
       <c r="E40" s="11">
-        <v>1051.2</v>
+        <v>1157.2</v>
       </c>
       <c r="F40" s="11">
-        <v>1176</v>
+        <v>1297.4</v>
       </c>
       <c r="G40" s="11">
-        <v>1261.4</v>
+        <v>1388.6</v>
       </c>
     </row>
     <row r="42" spans="1:7">
@@ -5772,22 +5774,22 @@
         <v>93</v>
       </c>
       <c r="B44">
-        <v>362</v>
+        <v>338</v>
       </c>
       <c r="C44">
-        <v>386</v>
+        <v>361</v>
       </c>
       <c r="D44">
-        <v>94.09999999999999</v>
+        <v>87.90000000000001</v>
       </c>
       <c r="E44">
-        <v>100.4</v>
+        <v>93.90000000000001</v>
       </c>
       <c r="F44">
-        <v>112.9</v>
+        <v>105.5</v>
       </c>
       <c r="G44">
-        <v>120.4</v>
+        <v>112.6</v>
       </c>
     </row>
     <row r="45" spans="1:7">
@@ -5795,22 +5797,22 @@
         <v>95</v>
       </c>
       <c r="B45">
-        <v>353</v>
+        <v>329</v>
       </c>
       <c r="C45">
-        <v>376</v>
+        <v>351</v>
       </c>
       <c r="D45">
-        <v>91.8</v>
+        <v>85.5</v>
       </c>
       <c r="E45">
-        <v>97.8</v>
+        <v>91.3</v>
       </c>
       <c r="F45">
-        <v>110.1</v>
+        <v>102.6</v>
       </c>
       <c r="G45">
-        <v>117.3</v>
+        <v>109.5</v>
       </c>
     </row>
     <row r="46" spans="1:7">
@@ -5818,22 +5820,22 @@
         <v>91</v>
       </c>
       <c r="B46">
+        <v>296</v>
+      </c>
+      <c r="C46">
         <v>317</v>
       </c>
-      <c r="C46">
-        <v>340</v>
-      </c>
       <c r="D46">
+        <v>77</v>
+      </c>
+      <c r="E46">
         <v>82.40000000000001</v>
       </c>
-      <c r="E46">
-        <v>88.40000000000001</v>
-      </c>
       <c r="F46">
+        <v>92.40000000000001</v>
+      </c>
+      <c r="G46">
         <v>98.90000000000001</v>
-      </c>
-      <c r="G46">
-        <v>106.1</v>
       </c>
     </row>
     <row r="47" spans="1:7">
@@ -5841,22 +5843,22 @@
         <v>103</v>
       </c>
       <c r="B47">
+        <v>275</v>
+      </c>
+      <c r="C47">
         <v>294</v>
       </c>
-      <c r="C47">
-        <v>315</v>
-      </c>
       <c r="D47">
+        <v>71.5</v>
+      </c>
+      <c r="E47">
         <v>76.40000000000001</v>
       </c>
-      <c r="E47">
-        <v>81.90000000000001</v>
-      </c>
       <c r="F47">
+        <v>85.8</v>
+      </c>
+      <c r="G47">
         <v>91.7</v>
-      </c>
-      <c r="G47">
-        <v>98.3</v>
       </c>
     </row>
     <row r="48" spans="1:7">
@@ -5864,22 +5866,22 @@
         <v>94</v>
       </c>
       <c r="B48">
-        <v>283</v>
+        <v>265</v>
       </c>
       <c r="C48">
-        <v>302</v>
+        <v>284</v>
       </c>
       <c r="D48">
-        <v>73.59999999999999</v>
+        <v>68.90000000000001</v>
       </c>
       <c r="E48">
-        <v>78.5</v>
+        <v>73.8</v>
       </c>
       <c r="F48">
-        <v>88.3</v>
+        <v>82.7</v>
       </c>
       <c r="G48">
-        <v>94.2</v>
+        <v>88.59999999999999</v>
       </c>
     </row>
     <row r="49" spans="1:7">
@@ -5887,22 +5889,22 @@
         <v>97</v>
       </c>
       <c r="B49">
-        <v>263</v>
+        <v>244</v>
       </c>
       <c r="C49">
-        <v>282</v>
+        <v>260</v>
       </c>
       <c r="D49">
-        <v>68.40000000000001</v>
+        <v>63.4</v>
       </c>
       <c r="E49">
-        <v>73.3</v>
+        <v>67.59999999999999</v>
       </c>
       <c r="F49">
-        <v>82.09999999999999</v>
+        <v>76.09999999999999</v>
       </c>
       <c r="G49">
-        <v>88</v>
+        <v>81.09999999999999</v>
       </c>
     </row>
     <row r="50" spans="1:7">
@@ -5910,22 +5912,22 @@
         <v>92</v>
       </c>
       <c r="B50">
-        <v>223</v>
+        <v>208</v>
       </c>
       <c r="C50">
-        <v>240</v>
+        <v>224</v>
       </c>
       <c r="D50">
-        <v>58</v>
+        <v>54.1</v>
       </c>
       <c r="E50">
-        <v>62.4</v>
+        <v>58.2</v>
       </c>
       <c r="F50">
-        <v>69.59999999999999</v>
+        <v>64.90000000000001</v>
       </c>
       <c r="G50">
-        <v>74.90000000000001</v>
+        <v>69.90000000000001</v>
       </c>
     </row>
     <row r="51" spans="1:7">
@@ -5933,22 +5935,22 @@
         <v>104</v>
       </c>
       <c r="B51">
-        <v>213</v>
+        <v>197</v>
       </c>
       <c r="C51">
-        <v>229</v>
+        <v>212</v>
       </c>
       <c r="D51">
-        <v>55.4</v>
+        <v>51.2</v>
       </c>
       <c r="E51">
-        <v>59.5</v>
+        <v>55.1</v>
       </c>
       <c r="F51">
-        <v>66.5</v>
+        <v>61.5</v>
       </c>
       <c r="G51">
-        <v>71.40000000000001</v>
+        <v>66.09999999999999</v>
       </c>
     </row>
     <row r="52" spans="1:7">
@@ -5956,22 +5958,22 @@
         <v>99</v>
       </c>
       <c r="B52">
-        <v>213</v>
+        <v>199</v>
       </c>
       <c r="C52">
-        <v>230</v>
+        <v>215</v>
       </c>
       <c r="D52">
-        <v>55.4</v>
+        <v>51.7</v>
       </c>
       <c r="E52">
-        <v>59.8</v>
+        <v>55.9</v>
       </c>
       <c r="F52">
-        <v>66.5</v>
+        <v>62.1</v>
       </c>
       <c r="G52">
-        <v>71.8</v>
+        <v>67.09999999999999</v>
       </c>
     </row>
     <row r="53" spans="1:7">
@@ -5979,22 +5981,22 @@
         <v>96</v>
       </c>
       <c r="B53">
-        <v>159</v>
+        <v>150</v>
       </c>
       <c r="C53">
-        <v>172</v>
+        <v>162</v>
       </c>
       <c r="D53">
-        <v>41.3</v>
+        <v>39</v>
       </c>
       <c r="E53">
-        <v>44.7</v>
+        <v>42.1</v>
       </c>
       <c r="F53">
-        <v>49.6</v>
+        <v>46.8</v>
       </c>
       <c r="G53">
-        <v>53.7</v>
+        <v>50.5</v>
       </c>
     </row>
     <row r="54" spans="1:7">
@@ -6002,22 +6004,22 @@
         <v>105</v>
       </c>
       <c r="B54">
-        <v>141</v>
+        <v>130</v>
       </c>
       <c r="C54">
-        <v>153</v>
+        <v>142</v>
       </c>
       <c r="D54">
-        <v>36.7</v>
+        <v>33.8</v>
       </c>
       <c r="E54">
-        <v>39.8</v>
+        <v>36.9</v>
       </c>
       <c r="F54">
-        <v>44</v>
+        <v>40.6</v>
       </c>
       <c r="G54">
-        <v>47.7</v>
+        <v>44.3</v>
       </c>
     </row>
     <row r="55" spans="1:7">
@@ -6025,22 +6027,22 @@
         <v>101</v>
       </c>
       <c r="B55">
-        <v>129</v>
+        <v>120</v>
       </c>
       <c r="C55">
-        <v>140</v>
+        <v>130</v>
       </c>
       <c r="D55">
-        <v>33.5</v>
+        <v>31.2</v>
       </c>
       <c r="E55">
-        <v>36.4</v>
+        <v>33.8</v>
       </c>
       <c r="F55">
-        <v>40.2</v>
+        <v>37.4</v>
       </c>
       <c r="G55">
-        <v>43.7</v>
+        <v>40.6</v>
       </c>
     </row>
     <row r="56" spans="1:7">
@@ -6048,22 +6050,22 @@
         <v>156</v>
       </c>
       <c r="B56" s="11">
-        <v>2950</v>
+        <v>2751</v>
       </c>
       <c r="C56" s="11">
-        <v>3165</v>
+        <v>2952</v>
       </c>
       <c r="D56" s="11">
-        <v>767</v>
+        <v>715.3</v>
       </c>
       <c r="E56" s="11">
-        <v>822.9</v>
+        <v>767.5</v>
       </c>
       <c r="F56" s="11">
-        <v>920.4</v>
+        <v>858.3</v>
       </c>
       <c r="G56" s="11">
-        <v>987.5</v>
+        <v>921</v>
       </c>
     </row>
   </sheetData>
@@ -6104,140 +6106,140 @@
       <c r="A5" t="s">
         <v>24</v>
       </c>
-      <c r="B5" s="8">
+      <c r="B5" s="12">
         <v>0.1841</v>
       </c>
       <c r="C5" s="9">
-        <v>488</v>
+        <v>478</v>
       </c>
       <c r="D5" s="9">
-        <v>522</v>
+        <v>512</v>
       </c>
     </row>
     <row r="6" spans="1:4">
       <c r="A6" t="s">
         <v>25</v>
       </c>
-      <c r="B6" s="8">
+      <c r="B6" s="12">
         <v>0.141</v>
       </c>
       <c r="C6" s="9">
-        <v>374</v>
+        <v>366</v>
       </c>
       <c r="D6" s="9">
-        <v>400</v>
+        <v>392</v>
       </c>
     </row>
     <row r="7" spans="1:4">
       <c r="A7" t="s">
         <v>26</v>
       </c>
-      <c r="B7" s="8">
+      <c r="B7" s="12">
         <v>0.141</v>
       </c>
       <c r="C7" s="9">
-        <v>374</v>
+        <v>366</v>
       </c>
       <c r="D7" s="9">
-        <v>400</v>
+        <v>392</v>
       </c>
     </row>
     <row r="8" spans="1:4">
       <c r="A8" t="s">
         <v>27</v>
       </c>
-      <c r="B8" s="8">
+      <c r="B8" s="12">
         <v>0.1289</v>
       </c>
       <c r="C8" s="9">
-        <v>342</v>
+        <v>335</v>
       </c>
       <c r="D8" s="9">
-        <v>366</v>
+        <v>359</v>
       </c>
     </row>
     <row r="9" spans="1:4">
       <c r="A9" t="s">
         <v>28</v>
       </c>
-      <c r="B9" s="8">
+      <c r="B9" s="12">
         <v>0.0202</v>
       </c>
       <c r="C9" s="9">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="D9" s="9">
-        <v>57</v>
+        <v>56</v>
       </c>
     </row>
     <row r="10" spans="1:4">
       <c r="A10" t="s">
         <v>29</v>
       </c>
-      <c r="B10" s="8">
+      <c r="B10" s="12">
         <v>0.141</v>
       </c>
       <c r="C10" s="9">
-        <v>374</v>
+        <v>366</v>
       </c>
       <c r="D10" s="9">
-        <v>400</v>
+        <v>392</v>
       </c>
     </row>
     <row r="11" spans="1:4">
       <c r="A11" t="s">
         <v>30</v>
       </c>
-      <c r="B11" s="8">
+      <c r="B11" s="12">
         <v>0.047</v>
       </c>
       <c r="C11" s="9">
-        <v>125</v>
+        <v>122</v>
       </c>
       <c r="D11" s="9">
-        <v>133</v>
+        <v>131</v>
       </c>
     </row>
     <row r="12" spans="1:4">
       <c r="A12" t="s">
         <v>31</v>
       </c>
-      <c r="B12" s="8">
+      <c r="B12" s="12">
         <v>0.092</v>
       </c>
       <c r="C12" s="9">
-        <v>244</v>
+        <v>239</v>
       </c>
       <c r="D12" s="9">
-        <v>261</v>
+        <v>256</v>
       </c>
     </row>
     <row r="13" spans="1:4">
       <c r="A13" t="s">
         <v>32</v>
       </c>
-      <c r="B13" s="8">
+      <c r="B13" s="12">
         <v>0.1048</v>
       </c>
       <c r="C13" s="9">
-        <v>278</v>
+        <v>272</v>
       </c>
       <c r="D13" s="9">
-        <v>297</v>
+        <v>292</v>
       </c>
     </row>
     <row r="14" spans="1:4">
-      <c r="A14" s="11" t="s">
+      <c r="A14" s="4" t="s">
         <v>77</v>
       </c>
-      <c r="B14" s="11">
+      <c r="B14" s="5">
         <v>1</v>
       </c>
-      <c r="C14" s="11">
-        <v>2653</v>
-      </c>
-      <c r="D14" s="11">
-        <v>2836</v>
+      <c r="C14" s="9">
+        <v>2596</v>
+      </c>
+      <c r="D14" s="9">
+        <v>2782</v>
       </c>
     </row>
     <row r="16" spans="1:4">
@@ -6263,140 +6265,140 @@
       <c r="A18" t="s">
         <v>24</v>
       </c>
-      <c r="B18" s="8">
+      <c r="B18" s="12">
         <v>0.2247</v>
       </c>
       <c r="C18" s="9">
-        <v>551</v>
+        <v>607</v>
       </c>
       <c r="D18" s="9">
-        <v>591</v>
+        <v>650</v>
       </c>
     </row>
     <row r="19" spans="1:4">
       <c r="A19" t="s">
         <v>25</v>
       </c>
-      <c r="B19" s="8">
+      <c r="B19" s="12">
         <v>0.1316</v>
       </c>
       <c r="C19" s="9">
-        <v>322</v>
+        <v>356</v>
       </c>
       <c r="D19" s="9">
-        <v>346</v>
+        <v>381</v>
       </c>
     </row>
     <row r="20" spans="1:4">
       <c r="A20" t="s">
         <v>26</v>
       </c>
-      <c r="B20" s="8">
+      <c r="B20" s="12">
         <v>0.1439</v>
       </c>
       <c r="C20" s="9">
-        <v>353</v>
+        <v>389</v>
       </c>
       <c r="D20" s="9">
-        <v>378</v>
+        <v>416</v>
       </c>
     </row>
     <row r="21" spans="1:4">
       <c r="A21" t="s">
         <v>27</v>
       </c>
-      <c r="B21" s="8">
+      <c r="B21" s="12">
         <v>0.093</v>
       </c>
       <c r="C21" s="9">
-        <v>228</v>
+        <v>251</v>
       </c>
       <c r="D21" s="9">
-        <v>244</v>
+        <v>269</v>
       </c>
     </row>
     <row r="22" spans="1:4">
       <c r="A22" t="s">
         <v>28</v>
       </c>
-      <c r="B22" s="8">
+      <c r="B22" s="12">
         <v>0.0119</v>
       </c>
       <c r="C22" s="9">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="D22" s="9">
-        <v>31</v>
+        <v>34</v>
       </c>
     </row>
     <row r="23" spans="1:4">
       <c r="A23" t="s">
         <v>29</v>
       </c>
-      <c r="B23" s="8">
+      <c r="B23" s="12">
         <v>0.1316</v>
       </c>
       <c r="C23" s="9">
-        <v>322</v>
+        <v>356</v>
       </c>
       <c r="D23" s="9">
-        <v>346</v>
+        <v>381</v>
       </c>
     </row>
     <row r="24" spans="1:4">
       <c r="A24" t="s">
         <v>30</v>
       </c>
-      <c r="B24" s="8">
+      <c r="B24" s="12">
         <v>0.0483</v>
       </c>
       <c r="C24" s="9">
-        <v>118</v>
+        <v>131</v>
       </c>
       <c r="D24" s="9">
-        <v>127</v>
+        <v>140</v>
       </c>
     </row>
     <row r="25" spans="1:4">
       <c r="A25" t="s">
         <v>31</v>
       </c>
-      <c r="B25" s="8">
+      <c r="B25" s="12">
         <v>0.1122</v>
       </c>
       <c r="C25" s="9">
-        <v>275</v>
+        <v>303</v>
       </c>
       <c r="D25" s="9">
-        <v>295</v>
+        <v>325</v>
       </c>
     </row>
     <row r="26" spans="1:4">
       <c r="A26" t="s">
         <v>32</v>
       </c>
-      <c r="B26" s="8">
+      <c r="B26" s="12">
         <v>0.1028</v>
       </c>
       <c r="C26" s="9">
-        <v>252</v>
+        <v>278</v>
       </c>
       <c r="D26" s="9">
-        <v>270</v>
+        <v>297</v>
       </c>
     </row>
     <row r="27" spans="1:4">
-      <c r="A27" s="11" t="s">
+      <c r="A27" s="4" t="s">
         <v>77</v>
       </c>
-      <c r="B27" s="11">
+      <c r="B27" s="5">
         <v>1</v>
       </c>
-      <c r="C27" s="11">
-        <v>2450</v>
-      </c>
-      <c r="D27" s="11">
-        <v>2628</v>
+      <c r="C27" s="9">
+        <v>2703</v>
+      </c>
+      <c r="D27" s="9">
+        <v>2893</v>
       </c>
     </row>
     <row r="29" spans="1:4">
@@ -6422,140 +6424,140 @@
       <c r="A31" t="s">
         <v>24</v>
       </c>
-      <c r="B31" s="8">
+      <c r="B31" s="12">
         <v>0.2022</v>
       </c>
       <c r="C31" s="9">
-        <v>596</v>
+        <v>556</v>
       </c>
       <c r="D31" s="9">
-        <v>640</v>
+        <v>597</v>
       </c>
     </row>
     <row r="32" spans="1:4">
       <c r="A32" t="s">
         <v>25</v>
       </c>
-      <c r="B32" s="8">
+      <c r="B32" s="12">
         <v>0.1338</v>
       </c>
       <c r="C32" s="9">
+        <v>368</v>
+      </c>
+      <c r="D32" s="9">
         <v>395</v>
-      </c>
-      <c r="D32" s="9">
-        <v>423</v>
       </c>
     </row>
     <row r="33" spans="1:4">
       <c r="A33" t="s">
         <v>26</v>
       </c>
-      <c r="B33" s="8">
+      <c r="B33" s="12">
         <v>0.1242</v>
       </c>
       <c r="C33" s="9">
-        <v>366</v>
+        <v>342</v>
       </c>
       <c r="D33" s="9">
-        <v>393</v>
+        <v>367</v>
       </c>
     </row>
     <row r="34" spans="1:4">
       <c r="A34" t="s">
         <v>27</v>
       </c>
-      <c r="B34" s="8">
+      <c r="B34" s="12">
         <v>0.1373</v>
       </c>
       <c r="C34" s="9">
+        <v>378</v>
+      </c>
+      <c r="D34" s="9">
         <v>405</v>
-      </c>
-      <c r="D34" s="9">
-        <v>435</v>
       </c>
     </row>
     <row r="35" spans="1:4">
       <c r="A35" t="s">
         <v>28</v>
       </c>
-      <c r="B35" s="8">
+      <c r="B35" s="12">
         <v>0.0406</v>
       </c>
       <c r="C35" s="9">
+        <v>112</v>
+      </c>
+      <c r="D35" s="9">
         <v>120</v>
-      </c>
-      <c r="D35" s="9">
-        <v>128</v>
       </c>
     </row>
     <row r="36" spans="1:4">
       <c r="A36" t="s">
         <v>29</v>
       </c>
-      <c r="B36" s="8">
+      <c r="B36" s="12">
         <v>0.1338</v>
       </c>
       <c r="C36" s="9">
+        <v>368</v>
+      </c>
+      <c r="D36" s="9">
         <v>395</v>
-      </c>
-      <c r="D36" s="9">
-        <v>423</v>
       </c>
     </row>
     <row r="37" spans="1:4">
       <c r="A37" t="s">
         <v>30</v>
       </c>
-      <c r="B37" s="8">
+      <c r="B37" s="12">
         <v>0.0333</v>
       </c>
       <c r="C37" s="9">
+        <v>92</v>
+      </c>
+      <c r="D37" s="9">
         <v>98</v>
-      </c>
-      <c r="D37" s="9">
-        <v>105</v>
       </c>
     </row>
     <row r="38" spans="1:4">
       <c r="A38" t="s">
         <v>31</v>
       </c>
-      <c r="B38" s="8">
+      <c r="B38" s="12">
         <v>0.1011</v>
       </c>
       <c r="C38" s="9">
+        <v>278</v>
+      </c>
+      <c r="D38" s="9">
         <v>298</v>
-      </c>
-      <c r="D38" s="9">
-        <v>320</v>
       </c>
     </row>
     <row r="39" spans="1:4">
       <c r="A39" t="s">
         <v>32</v>
       </c>
-      <c r="B39" s="8">
+      <c r="B39" s="12">
         <v>0.09379999999999999</v>
       </c>
       <c r="C39" s="9">
+        <v>258</v>
+      </c>
+      <c r="D39" s="9">
         <v>277</v>
       </c>
-      <c r="D39" s="9">
-        <v>297</v>
-      </c>
     </row>
     <row r="40" spans="1:4">
-      <c r="A40" s="11" t="s">
+      <c r="A40" s="4" t="s">
         <v>77</v>
       </c>
-      <c r="B40" s="11">
+      <c r="B40" s="5">
         <v>1</v>
       </c>
-      <c r="C40" s="11">
-        <v>2950</v>
-      </c>
-      <c r="D40" s="11">
-        <v>3164</v>
+      <c r="C40" s="9">
+        <v>2752</v>
+      </c>
+      <c r="D40" s="9">
+        <v>2952</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update Rio tela consumption: CAB 0.66, DAMA 0.52, KIDS 0.32 kg/und
Co-authored-by: scm-svg <scm-svg@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/RIO_ORIGINAL_Proyeccion_Produccion.xlsx
+++ b/RIO_ORIGINAL_Proyeccion_Produccion.xlsx
@@ -52,7 +52,7 @@
     <t>• Color: ventas históricas Oct–Ago · Talla: Jun–Ago · Stock actual referenciado en Resumen y dashboard.</t>
   </si>
   <si>
-    <t>• Tela Jabón Microfibra: consumo en kg/und (CAB 0.5 · DAMA 0.4 · KIDS 0.26).</t>
+    <t>• Tela Jabón Microfibra: consumo en kg/und (CAB 0.66 · DAMA 0.52 · KIDS 0.32).</t>
   </si>
   <si>
     <t>• Meta de producción: CAB 2,596 · DAMA 2,703 · KIDS 2,751 und (mínimo compromiso).</t>
@@ -457,7 +457,7 @@
     <t>Consumo (kg/und)</t>
   </si>
   <si>
-    <t>CABALLERO — COMPRA DE TELA POR COLOR (consumo 0.5 kg/und)</t>
+    <t>CABALLERO — COMPRA DE TELA POR COLOR (consumo 0.66 kg/und)</t>
   </si>
   <si>
     <t>Und Mín</t>
@@ -481,13 +481,13 @@
     <t>TOTAL CABALLERO</t>
   </si>
   <si>
-    <t>DAMA — COMPRA DE TELA POR COLOR (consumo 0.4 kg/und)</t>
+    <t>DAMA — COMPRA DE TELA POR COLOR (consumo 0.52 kg/und)</t>
   </si>
   <si>
     <t>TOTAL DAMA</t>
   </si>
   <si>
-    <t>KIDS — COMPRA DE TELA POR COLOR (consumo 0.26 kg/und)</t>
+    <t>KIDS — COMPRA DE TELA POR COLOR (consumo 0.32 kg/und)</t>
   </si>
   <si>
     <t>TOTAL KIDS</t>
@@ -520,7 +520,7 @@
     <t>• Colores activos para producción: catálogo Rio Original (11 CAB · 12 DAMA · 12 KIDS).</t>
   </si>
   <si>
-    <t>• Consumo tela Jabón Microfibra: CAB 0.5 kg/und · DAMA 0.4 kg/und · KIDS 0.26 kg/und.</t>
+    <t>• Consumo tela Jabón Microfibra: CAB 0.66 kg/und · DAMA 0.52 kg/und · KIDS 0.32 kg/und.</t>
   </si>
   <si>
     <t>2. VELOCIDAD BASE Y AJUSTES POR TIENDA</t>
@@ -587,12 +587,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="5">
+  <numFmts count="4">
     <numFmt numFmtId="164" formatCode="0%"/>
     <numFmt numFmtId="165" formatCode="0.0"/>
-    <numFmt numFmtId="166" formatCode="0.0000%"/>
+    <numFmt numFmtId="166" formatCode="0.00%"/>
     <numFmt numFmtId="167" formatCode="#,##0"/>
-    <numFmt numFmtId="168" formatCode="0.00%"/>
   </numFmts>
   <fonts count="5">
     <font>
@@ -691,7 +690,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -706,7 +705,6 @@
     <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="167" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1352,7 +1350,7 @@
       <c r="C33" s="7">
         <v>490.2</v>
       </c>
-      <c r="D33" s="8">
+      <c r="D33" s="5">
         <v>1</v>
       </c>
     </row>
@@ -1600,7 +1598,7 @@
       <c r="C57" s="7">
         <v>443.3</v>
       </c>
-      <c r="D57" s="8">
+      <c r="D57" s="5">
         <v>1</v>
       </c>
     </row>
@@ -1848,7 +1846,7 @@
       <c r="C81" s="7">
         <v>640.7</v>
       </c>
-      <c r="D81" s="8">
+      <c r="D81" s="5">
         <v>1</v>
       </c>
     </row>
@@ -2625,7 +2623,7 @@
       <c r="A5" t="s">
         <v>91</v>
       </c>
-      <c r="B5" s="12">
+      <c r="B5" s="8">
         <v>0.2014637904468413</v>
       </c>
       <c r="C5" s="9">
@@ -2639,7 +2637,7 @@
       <c r="A6" t="s">
         <v>92</v>
       </c>
-      <c r="B6" s="12">
+      <c r="B6" s="8">
         <v>0.1278890600924499</v>
       </c>
       <c r="C6" s="9">
@@ -2653,7 +2651,7 @@
       <c r="A7" t="s">
         <v>93</v>
       </c>
-      <c r="B7" s="12">
+      <c r="B7" s="8">
         <v>0.1209553158705701</v>
       </c>
       <c r="C7" s="9">
@@ -2667,7 +2665,7 @@
       <c r="A8" t="s">
         <v>94</v>
       </c>
-      <c r="B8" s="12">
+      <c r="B8" s="8">
         <v>0.09976887519260401</v>
       </c>
       <c r="C8" s="9">
@@ -2681,7 +2679,7 @@
       <c r="A9" t="s">
         <v>95</v>
       </c>
-      <c r="B9" s="12">
+      <c r="B9" s="8">
         <v>0.09591679506933744</v>
       </c>
       <c r="C9" s="9">
@@ -2695,7 +2693,7 @@
       <c r="A10" t="s">
         <v>96</v>
       </c>
-      <c r="B10" s="12">
+      <c r="B10" s="8">
         <v>0.08782742681047766</v>
       </c>
       <c r="C10" s="9">
@@ -2709,7 +2707,7 @@
       <c r="A11" t="s">
         <v>97</v>
       </c>
-      <c r="B11" s="12">
+      <c r="B11" s="8">
         <v>0.08166409861325115</v>
       </c>
       <c r="C11" s="9">
@@ -2723,7 +2721,7 @@
       <c r="A12" t="s">
         <v>98</v>
       </c>
-      <c r="B12" s="12">
+      <c r="B12" s="8">
         <v>0.06548536209553159</v>
       </c>
       <c r="C12" s="9">
@@ -2737,7 +2735,7 @@
       <c r="A13" t="s">
         <v>99</v>
       </c>
-      <c r="B13" s="12">
+      <c r="B13" s="8">
         <v>0.05508474576271186</v>
       </c>
       <c r="C13" s="9">
@@ -2751,7 +2749,7 @@
       <c r="A14" t="s">
         <v>100</v>
       </c>
-      <c r="B14" s="12">
+      <c r="B14" s="8">
         <v>0.04776579352850539</v>
       </c>
       <c r="C14" s="9">
@@ -2765,7 +2763,7 @@
       <c r="A15" t="s">
         <v>101</v>
       </c>
-      <c r="B15" s="12">
+      <c r="B15" s="8">
         <v>0.01617873651771957</v>
       </c>
       <c r="C15" s="9">
@@ -2812,7 +2810,7 @@
       <c r="A20" t="s">
         <v>91</v>
       </c>
-      <c r="B20" s="12">
+      <c r="B20" s="8">
         <v>0.1949685534591195</v>
       </c>
       <c r="C20" s="9">
@@ -2826,7 +2824,7 @@
       <c r="A21" t="s">
         <v>93</v>
       </c>
-      <c r="B21" s="12">
+      <c r="B21" s="8">
         <v>0.1342952275249722</v>
       </c>
       <c r="C21" s="9">
@@ -2840,7 +2838,7 @@
       <c r="A22" t="s">
         <v>92</v>
       </c>
-      <c r="B22" s="12">
+      <c r="B22" s="8">
         <v>0.1187569367369589</v>
       </c>
       <c r="C22" s="9">
@@ -2854,7 +2852,7 @@
       <c r="A23" t="s">
         <v>99</v>
       </c>
-      <c r="B23" s="12">
+      <c r="B23" s="8">
         <v>0.09914909359970403</v>
       </c>
       <c r="C23" s="9">
@@ -2868,7 +2866,7 @@
       <c r="A24" t="s">
         <v>103</v>
       </c>
-      <c r="B24" s="12">
+      <c r="B24" s="8">
         <v>0.09766925638179801</v>
       </c>
       <c r="C24" s="9">
@@ -2882,7 +2880,7 @@
       <c r="A25" t="s">
         <v>95</v>
       </c>
-      <c r="B25" s="12">
+      <c r="B25" s="8">
         <v>0.09322974472807991</v>
       </c>
       <c r="C25" s="9">
@@ -2896,7 +2894,7 @@
       <c r="A26" t="s">
         <v>97</v>
       </c>
-      <c r="B26" s="12">
+      <c r="B26" s="8">
         <v>0.06215316315205328</v>
       </c>
       <c r="C26" s="9">
@@ -2910,7 +2908,7 @@
       <c r="A27" t="s">
         <v>98</v>
       </c>
-      <c r="B27" s="12">
+      <c r="B27" s="8">
         <v>0.05623381428042915</v>
       </c>
       <c r="C27" s="9">
@@ -2924,7 +2922,7 @@
       <c r="A28" t="s">
         <v>96</v>
       </c>
-      <c r="B28" s="12">
+      <c r="B28" s="8">
         <v>0.04994450610432852</v>
       </c>
       <c r="C28" s="9">
@@ -2938,7 +2936,7 @@
       <c r="A29" t="s">
         <v>104</v>
       </c>
-      <c r="B29" s="12">
+      <c r="B29" s="8">
         <v>0.04809470958194598</v>
       </c>
       <c r="C29" s="9">
@@ -2952,7 +2950,7 @@
       <c r="A30" t="s">
         <v>105</v>
       </c>
-      <c r="B30" s="12">
+      <c r="B30" s="8">
         <v>0.0244173140954495</v>
       </c>
       <c r="C30" s="9">
@@ -2966,7 +2964,7 @@
       <c r="A31" t="s">
         <v>101</v>
       </c>
-      <c r="B31" s="12">
+      <c r="B31" s="8">
         <v>0.02108768035516093</v>
       </c>
       <c r="C31" s="9">
@@ -3013,7 +3011,7 @@
       <c r="A36" t="s">
         <v>93</v>
       </c>
-      <c r="B36" s="12">
+      <c r="B36" s="8">
         <v>0.1228644129407488</v>
       </c>
       <c r="C36" s="9">
@@ -3027,7 +3025,7 @@
       <c r="A37" t="s">
         <v>95</v>
       </c>
-      <c r="B37" s="12">
+      <c r="B37" s="8">
         <v>0.1195928753180662</v>
       </c>
       <c r="C37" s="9">
@@ -3041,7 +3039,7 @@
       <c r="A38" t="s">
         <v>91</v>
       </c>
-      <c r="B38" s="12">
+      <c r="B38" s="8">
         <v>0.1075972373682297</v>
       </c>
       <c r="C38" s="9">
@@ -3055,7 +3053,7 @@
       <c r="A39" t="s">
         <v>103</v>
       </c>
-      <c r="B39" s="12">
+      <c r="B39" s="8">
         <v>0.0999636495819702</v>
       </c>
       <c r="C39" s="9">
@@ -3069,7 +3067,7 @@
       <c r="A40" t="s">
         <v>94</v>
       </c>
-      <c r="B40" s="12">
+      <c r="B40" s="8">
         <v>0.09632860777898945</v>
       </c>
       <c r="C40" s="9">
@@ -3083,7 +3081,7 @@
       <c r="A41" t="s">
         <v>97</v>
       </c>
-      <c r="B41" s="12">
+      <c r="B41" s="8">
         <v>0.08869501999272991</v>
       </c>
       <c r="C41" s="9">
@@ -3097,7 +3095,7 @@
       <c r="A42" t="s">
         <v>92</v>
       </c>
-      <c r="B42" s="12">
+      <c r="B42" s="8">
         <v>0.07560886950199927</v>
       </c>
       <c r="C42" s="9">
@@ -3111,7 +3109,7 @@
       <c r="A43" t="s">
         <v>104</v>
       </c>
-      <c r="B43" s="12">
+      <c r="B43" s="8">
         <v>0.07161032351872046</v>
       </c>
       <c r="C43" s="9">
@@ -3125,7 +3123,7 @@
       <c r="A44" t="s">
         <v>99</v>
       </c>
-      <c r="B44" s="12">
+      <c r="B44" s="8">
         <v>0.07233733187931661</v>
       </c>
       <c r="C44" s="9">
@@ -3139,7 +3137,7 @@
       <c r="A45" t="s">
         <v>96</v>
       </c>
-      <c r="B45" s="12">
+      <c r="B45" s="8">
         <v>0.05452562704471101</v>
       </c>
       <c r="C45" s="9">
@@ -3153,7 +3151,7 @@
       <c r="A46" t="s">
         <v>105</v>
       </c>
-      <c r="B46" s="12">
+      <c r="B46" s="8">
         <v>0.04725554343874955</v>
       </c>
       <c r="C46" s="9">
@@ -3167,7 +3165,7 @@
       <c r="A47" t="s">
         <v>101</v>
       </c>
-      <c r="B47" s="12">
+      <c r="B47" s="8">
         <v>0.04362050163576881</v>
       </c>
       <c r="C47" s="9">
@@ -5091,7 +5089,7 @@
         <v>47</v>
       </c>
       <c r="B7">
-        <v>0.5</v>
+        <v>0.66</v>
       </c>
     </row>
     <row r="8" spans="1:7">
@@ -5099,7 +5097,7 @@
         <v>48</v>
       </c>
       <c r="B8">
-        <v>0.4</v>
+        <v>0.52</v>
       </c>
     </row>
     <row r="9" spans="1:7">
@@ -5107,7 +5105,7 @@
         <v>49</v>
       </c>
       <c r="B9">
-        <v>0.26</v>
+        <v>0.32</v>
       </c>
     </row>
     <row r="11" spans="1:7">
@@ -5149,16 +5147,16 @@
         <v>557</v>
       </c>
       <c r="D13">
-        <v>261.5</v>
+        <v>345.2</v>
       </c>
       <c r="E13">
-        <v>278.5</v>
+        <v>367.6</v>
       </c>
       <c r="F13">
-        <v>313.8</v>
+        <v>414.2</v>
       </c>
       <c r="G13">
-        <v>334.2</v>
+        <v>441.1</v>
       </c>
     </row>
     <row r="14" spans="1:7">
@@ -5172,16 +5170,16 @@
         <v>356</v>
       </c>
       <c r="D14">
-        <v>166</v>
+        <v>219.1</v>
       </c>
       <c r="E14">
-        <v>178</v>
+        <v>235</v>
       </c>
       <c r="F14">
-        <v>199.2</v>
+        <v>262.9</v>
       </c>
       <c r="G14">
-        <v>213.6</v>
+        <v>282</v>
       </c>
     </row>
     <row r="15" spans="1:7">
@@ -5195,16 +5193,16 @@
         <v>336</v>
       </c>
       <c r="D15">
-        <v>157</v>
+        <v>207.2</v>
       </c>
       <c r="E15">
-        <v>168</v>
+        <v>221.8</v>
       </c>
       <c r="F15">
-        <v>188.4</v>
+        <v>248.7</v>
       </c>
       <c r="G15">
-        <v>201.6</v>
+        <v>266.1</v>
       </c>
     </row>
     <row r="16" spans="1:7">
@@ -5218,16 +5216,16 @@
         <v>277</v>
       </c>
       <c r="D16">
-        <v>129.5</v>
+        <v>170.9</v>
       </c>
       <c r="E16">
-        <v>138.5</v>
+        <v>182.8</v>
       </c>
       <c r="F16">
-        <v>155.4</v>
+        <v>205.1</v>
       </c>
       <c r="G16">
-        <v>166.2</v>
+        <v>219.4</v>
       </c>
     </row>
     <row r="17" spans="1:7">
@@ -5241,16 +5239,16 @@
         <v>267</v>
       </c>
       <c r="D17">
-        <v>124.5</v>
+        <v>164.3</v>
       </c>
       <c r="E17">
-        <v>133.5</v>
+        <v>176.2</v>
       </c>
       <c r="F17">
-        <v>149.4</v>
+        <v>197.2</v>
       </c>
       <c r="G17">
-        <v>160.2</v>
+        <v>211.5</v>
       </c>
     </row>
     <row r="18" spans="1:7">
@@ -5264,16 +5262,16 @@
         <v>245</v>
       </c>
       <c r="D18">
-        <v>114</v>
+        <v>150.5</v>
       </c>
       <c r="E18">
-        <v>122.5</v>
+        <v>161.7</v>
       </c>
       <c r="F18">
-        <v>136.8</v>
+        <v>180.6</v>
       </c>
       <c r="G18">
-        <v>147</v>
+        <v>194</v>
       </c>
     </row>
     <row r="19" spans="1:7">
@@ -5287,16 +5285,16 @@
         <v>227</v>
       </c>
       <c r="D19">
-        <v>106</v>
+        <v>139.9</v>
       </c>
       <c r="E19">
-        <v>113.5</v>
+        <v>149.8</v>
       </c>
       <c r="F19">
-        <v>127.2</v>
+        <v>167.9</v>
       </c>
       <c r="G19">
-        <v>136.2</v>
+        <v>179.8</v>
       </c>
     </row>
     <row r="20" spans="1:7">
@@ -5310,16 +5308,16 @@
         <v>183</v>
       </c>
       <c r="D20">
-        <v>85</v>
+        <v>112.2</v>
       </c>
       <c r="E20">
-        <v>91.5</v>
+        <v>120.8</v>
       </c>
       <c r="F20">
-        <v>102</v>
+        <v>134.6</v>
       </c>
       <c r="G20">
-        <v>109.8</v>
+        <v>144.9</v>
       </c>
     </row>
     <row r="21" spans="1:7">
@@ -5333,16 +5331,16 @@
         <v>154</v>
       </c>
       <c r="D21">
-        <v>71.5</v>
+        <v>94.40000000000001</v>
       </c>
       <c r="E21">
-        <v>77</v>
+        <v>101.6</v>
       </c>
       <c r="F21">
-        <v>85.8</v>
+        <v>113.3</v>
       </c>
       <c r="G21">
-        <v>92.40000000000001</v>
+        <v>122</v>
       </c>
     </row>
     <row r="22" spans="1:7">
@@ -5356,16 +5354,16 @@
         <v>133</v>
       </c>
       <c r="D22">
-        <v>62</v>
+        <v>81.8</v>
       </c>
       <c r="E22">
-        <v>66.5</v>
+        <v>87.8</v>
       </c>
       <c r="F22">
-        <v>74.40000000000001</v>
+        <v>98.2</v>
       </c>
       <c r="G22">
-        <v>79.8</v>
+        <v>105.3</v>
       </c>
     </row>
     <row r="23" spans="1:7">
@@ -5379,16 +5377,16 @@
         <v>47</v>
       </c>
       <c r="D23">
-        <v>21</v>
+        <v>27.7</v>
       </c>
       <c r="E23">
-        <v>23.5</v>
+        <v>31</v>
       </c>
       <c r="F23">
-        <v>25.2</v>
+        <v>33.3</v>
       </c>
       <c r="G23">
-        <v>28.2</v>
+        <v>37.2</v>
       </c>
     </row>
     <row r="24" spans="1:7">
@@ -5402,16 +5400,16 @@
         <v>2782</v>
       </c>
       <c r="D24" s="11">
-        <v>1298</v>
+        <v>1713.4</v>
       </c>
       <c r="E24" s="11">
-        <v>1391</v>
+        <v>1836.1</v>
       </c>
       <c r="F24" s="11">
-        <v>1557.6</v>
+        <v>2056</v>
       </c>
       <c r="G24" s="11">
-        <v>1669.2</v>
+        <v>2203.3</v>
       </c>
     </row>
     <row r="26" spans="1:7">
@@ -5453,16 +5451,16 @@
         <v>561</v>
       </c>
       <c r="D28">
-        <v>210.8</v>
+        <v>274</v>
       </c>
       <c r="E28">
-        <v>224.4</v>
+        <v>291.7</v>
       </c>
       <c r="F28">
-        <v>253</v>
+        <v>328.8</v>
       </c>
       <c r="G28">
-        <v>269.3</v>
+        <v>350.1</v>
       </c>
     </row>
     <row r="29" spans="1:7">
@@ -5476,16 +5474,16 @@
         <v>388</v>
       </c>
       <c r="D29">
-        <v>145.2</v>
+        <v>188.8</v>
       </c>
       <c r="E29">
-        <v>155.2</v>
+        <v>201.8</v>
       </c>
       <c r="F29">
-        <v>174.2</v>
+        <v>226.5</v>
       </c>
       <c r="G29">
-        <v>186.2</v>
+        <v>242.1</v>
       </c>
     </row>
     <row r="30" spans="1:7">
@@ -5499,16 +5497,16 @@
         <v>343</v>
       </c>
       <c r="D30">
-        <v>128.4</v>
+        <v>166.9</v>
       </c>
       <c r="E30">
-        <v>137.2</v>
+        <v>178.4</v>
       </c>
       <c r="F30">
-        <v>154.1</v>
+        <v>200.3</v>
       </c>
       <c r="G30">
-        <v>164.6</v>
+        <v>214</v>
       </c>
     </row>
     <row r="31" spans="1:7">
@@ -5522,16 +5520,16 @@
         <v>286</v>
       </c>
       <c r="D31">
-        <v>107.2</v>
+        <v>139.4</v>
       </c>
       <c r="E31">
-        <v>114.4</v>
+        <v>148.7</v>
       </c>
       <c r="F31">
-        <v>128.6</v>
+        <v>167.2</v>
       </c>
       <c r="G31">
-        <v>137.3</v>
+        <v>178.5</v>
       </c>
     </row>
     <row r="32" spans="1:7">
@@ -5545,16 +5543,16 @@
         <v>283</v>
       </c>
       <c r="D32">
-        <v>105.6</v>
+        <v>137.3</v>
       </c>
       <c r="E32">
-        <v>113.2</v>
+        <v>147.2</v>
       </c>
       <c r="F32">
-        <v>126.7</v>
+        <v>164.7</v>
       </c>
       <c r="G32">
-        <v>135.8</v>
+        <v>176.6</v>
       </c>
     </row>
     <row r="33" spans="1:7">
@@ -5568,16 +5566,16 @@
         <v>269</v>
       </c>
       <c r="D33">
-        <v>100.8</v>
+        <v>131</v>
       </c>
       <c r="E33">
-        <v>107.6</v>
+        <v>139.9</v>
       </c>
       <c r="F33">
-        <v>121</v>
+        <v>157.2</v>
       </c>
       <c r="G33">
-        <v>129.1</v>
+        <v>167.9</v>
       </c>
     </row>
     <row r="34" spans="1:7">
@@ -5591,16 +5589,16 @@
         <v>180</v>
       </c>
       <c r="D34">
-        <v>67.2</v>
+        <v>87.40000000000001</v>
       </c>
       <c r="E34">
-        <v>72</v>
+        <v>93.59999999999999</v>
       </c>
       <c r="F34">
-        <v>80.59999999999999</v>
+        <v>104.8</v>
       </c>
       <c r="G34">
-        <v>86.40000000000001</v>
+        <v>112.3</v>
       </c>
     </row>
     <row r="35" spans="1:7">
@@ -5614,16 +5612,16 @@
         <v>163</v>
       </c>
       <c r="D35">
-        <v>60.8</v>
+        <v>79</v>
       </c>
       <c r="E35">
-        <v>65.2</v>
+        <v>84.8</v>
       </c>
       <c r="F35">
-        <v>73</v>
+        <v>94.8</v>
       </c>
       <c r="G35">
-        <v>78.2</v>
+        <v>101.7</v>
       </c>
     </row>
     <row r="36" spans="1:7">
@@ -5637,16 +5635,16 @@
         <v>146</v>
       </c>
       <c r="D36">
-        <v>54</v>
+        <v>70.2</v>
       </c>
       <c r="E36">
-        <v>58.4</v>
+        <v>75.90000000000001</v>
       </c>
       <c r="F36">
-        <v>64.8</v>
+        <v>84.2</v>
       </c>
       <c r="G36">
-        <v>70.09999999999999</v>
+        <v>91.09999999999999</v>
       </c>
     </row>
     <row r="37" spans="1:7">
@@ -5660,16 +5658,16 @@
         <v>140</v>
       </c>
       <c r="D37">
-        <v>52</v>
+        <v>67.59999999999999</v>
       </c>
       <c r="E37">
-        <v>56</v>
+        <v>72.8</v>
       </c>
       <c r="F37">
-        <v>62.4</v>
+        <v>81.09999999999999</v>
       </c>
       <c r="G37">
-        <v>67.2</v>
+        <v>87.40000000000001</v>
       </c>
     </row>
     <row r="38" spans="1:7">
@@ -5683,16 +5681,16 @@
         <v>72</v>
       </c>
       <c r="D38">
-        <v>26.4</v>
+        <v>34.3</v>
       </c>
       <c r="E38">
-        <v>28.8</v>
+        <v>37.4</v>
       </c>
       <c r="F38">
-        <v>31.7</v>
+        <v>41.2</v>
       </c>
       <c r="G38">
-        <v>34.6</v>
+        <v>44.9</v>
       </c>
     </row>
     <row r="39" spans="1:7">
@@ -5706,16 +5704,16 @@
         <v>62</v>
       </c>
       <c r="D39">
-        <v>22.8</v>
+        <v>29.6</v>
       </c>
       <c r="E39">
-        <v>24.8</v>
+        <v>32.2</v>
       </c>
       <c r="F39">
-        <v>27.4</v>
+        <v>35.6</v>
       </c>
       <c r="G39">
-        <v>29.8</v>
+        <v>38.7</v>
       </c>
     </row>
     <row r="40" spans="1:7">
@@ -5729,16 +5727,16 @@
         <v>2893</v>
       </c>
       <c r="D40" s="11">
-        <v>1081.2</v>
+        <v>1405.6</v>
       </c>
       <c r="E40" s="11">
-        <v>1157.2</v>
+        <v>1504.4</v>
       </c>
       <c r="F40" s="11">
-        <v>1297.4</v>
+        <v>1686.7</v>
       </c>
       <c r="G40" s="11">
-        <v>1388.6</v>
+        <v>1805.2</v>
       </c>
     </row>
     <row r="42" spans="1:7">
@@ -5780,16 +5778,16 @@
         <v>361</v>
       </c>
       <c r="D44">
-        <v>87.90000000000001</v>
+        <v>108.2</v>
       </c>
       <c r="E44">
-        <v>93.90000000000001</v>
+        <v>115.5</v>
       </c>
       <c r="F44">
-        <v>105.5</v>
+        <v>129.8</v>
       </c>
       <c r="G44">
-        <v>112.6</v>
+        <v>138.6</v>
       </c>
     </row>
     <row r="45" spans="1:7">
@@ -5803,16 +5801,16 @@
         <v>351</v>
       </c>
       <c r="D45">
-        <v>85.5</v>
+        <v>105.3</v>
       </c>
       <c r="E45">
-        <v>91.3</v>
+        <v>112.3</v>
       </c>
       <c r="F45">
-        <v>102.6</v>
+        <v>126.3</v>
       </c>
       <c r="G45">
-        <v>109.5</v>
+        <v>134.8</v>
       </c>
     </row>
     <row r="46" spans="1:7">
@@ -5826,16 +5824,16 @@
         <v>317</v>
       </c>
       <c r="D46">
-        <v>77</v>
+        <v>94.7</v>
       </c>
       <c r="E46">
-        <v>82.40000000000001</v>
+        <v>101.4</v>
       </c>
       <c r="F46">
-        <v>92.40000000000001</v>
+        <v>113.7</v>
       </c>
       <c r="G46">
-        <v>98.90000000000001</v>
+        <v>121.7</v>
       </c>
     </row>
     <row r="47" spans="1:7">
@@ -5849,16 +5847,16 @@
         <v>294</v>
       </c>
       <c r="D47">
-        <v>71.5</v>
+        <v>88</v>
       </c>
       <c r="E47">
-        <v>76.40000000000001</v>
+        <v>94.09999999999999</v>
       </c>
       <c r="F47">
-        <v>85.8</v>
+        <v>105.6</v>
       </c>
       <c r="G47">
-        <v>91.7</v>
+        <v>112.9</v>
       </c>
     </row>
     <row r="48" spans="1:7">
@@ -5872,16 +5870,16 @@
         <v>284</v>
       </c>
       <c r="D48">
-        <v>68.90000000000001</v>
+        <v>84.8</v>
       </c>
       <c r="E48">
-        <v>73.8</v>
+        <v>90.90000000000001</v>
       </c>
       <c r="F48">
-        <v>82.7</v>
+        <v>101.8</v>
       </c>
       <c r="G48">
-        <v>88.59999999999999</v>
+        <v>109.1</v>
       </c>
     </row>
     <row r="49" spans="1:7">
@@ -5895,16 +5893,16 @@
         <v>260</v>
       </c>
       <c r="D49">
-        <v>63.4</v>
+        <v>78.09999999999999</v>
       </c>
       <c r="E49">
-        <v>67.59999999999999</v>
+        <v>83.2</v>
       </c>
       <c r="F49">
-        <v>76.09999999999999</v>
+        <v>93.7</v>
       </c>
       <c r="G49">
-        <v>81.09999999999999</v>
+        <v>99.8</v>
       </c>
     </row>
     <row r="50" spans="1:7">
@@ -5918,16 +5916,16 @@
         <v>224</v>
       </c>
       <c r="D50">
-        <v>54.1</v>
+        <v>66.59999999999999</v>
       </c>
       <c r="E50">
-        <v>58.2</v>
+        <v>71.7</v>
       </c>
       <c r="F50">
-        <v>64.90000000000001</v>
+        <v>79.90000000000001</v>
       </c>
       <c r="G50">
-        <v>69.90000000000001</v>
+        <v>86</v>
       </c>
     </row>
     <row r="51" spans="1:7">
@@ -5941,16 +5939,16 @@
         <v>212</v>
       </c>
       <c r="D51">
-        <v>51.2</v>
+        <v>63</v>
       </c>
       <c r="E51">
-        <v>55.1</v>
+        <v>67.8</v>
       </c>
       <c r="F51">
-        <v>61.5</v>
+        <v>75.59999999999999</v>
       </c>
       <c r="G51">
-        <v>66.09999999999999</v>
+        <v>81.40000000000001</v>
       </c>
     </row>
     <row r="52" spans="1:7">
@@ -5964,16 +5962,16 @@
         <v>215</v>
       </c>
       <c r="D52">
-        <v>51.7</v>
+        <v>63.7</v>
       </c>
       <c r="E52">
-        <v>55.9</v>
+        <v>68.8</v>
       </c>
       <c r="F52">
-        <v>62.1</v>
+        <v>76.40000000000001</v>
       </c>
       <c r="G52">
-        <v>67.09999999999999</v>
+        <v>82.59999999999999</v>
       </c>
     </row>
     <row r="53" spans="1:7">
@@ -5987,16 +5985,16 @@
         <v>162</v>
       </c>
       <c r="D53">
-        <v>39</v>
+        <v>48</v>
       </c>
       <c r="E53">
-        <v>42.1</v>
+        <v>51.8</v>
       </c>
       <c r="F53">
-        <v>46.8</v>
+        <v>57.6</v>
       </c>
       <c r="G53">
-        <v>50.5</v>
+        <v>62.2</v>
       </c>
     </row>
     <row r="54" spans="1:7">
@@ -6010,16 +6008,16 @@
         <v>142</v>
       </c>
       <c r="D54">
-        <v>33.8</v>
+        <v>41.6</v>
       </c>
       <c r="E54">
-        <v>36.9</v>
+        <v>45.4</v>
       </c>
       <c r="F54">
-        <v>40.6</v>
+        <v>49.9</v>
       </c>
       <c r="G54">
-        <v>44.3</v>
+        <v>54.5</v>
       </c>
     </row>
     <row r="55" spans="1:7">
@@ -6033,16 +6031,16 @@
         <v>130</v>
       </c>
       <c r="D55">
-        <v>31.2</v>
+        <v>38.4</v>
       </c>
       <c r="E55">
-        <v>33.8</v>
+        <v>41.6</v>
       </c>
       <c r="F55">
-        <v>37.4</v>
+        <v>46.1</v>
       </c>
       <c r="G55">
-        <v>40.6</v>
+        <v>49.9</v>
       </c>
     </row>
     <row r="56" spans="1:7">
@@ -6056,16 +6054,16 @@
         <v>2952</v>
       </c>
       <c r="D56" s="11">
-        <v>715.3</v>
+        <v>880.3</v>
       </c>
       <c r="E56" s="11">
-        <v>767.5</v>
+        <v>944.6</v>
       </c>
       <c r="F56" s="11">
-        <v>858.3</v>
+        <v>1056.4</v>
       </c>
       <c r="G56" s="11">
-        <v>921</v>
+        <v>1133.6</v>
       </c>
     </row>
   </sheetData>
@@ -6106,7 +6104,7 @@
       <c r="A5" t="s">
         <v>24</v>
       </c>
-      <c r="B5" s="12">
+      <c r="B5" s="8">
         <v>0.1841</v>
       </c>
       <c r="C5" s="9">
@@ -6120,7 +6118,7 @@
       <c r="A6" t="s">
         <v>25</v>
       </c>
-      <c r="B6" s="12">
+      <c r="B6" s="8">
         <v>0.141</v>
       </c>
       <c r="C6" s="9">
@@ -6134,7 +6132,7 @@
       <c r="A7" t="s">
         <v>26</v>
       </c>
-      <c r="B7" s="12">
+      <c r="B7" s="8">
         <v>0.141</v>
       </c>
       <c r="C7" s="9">
@@ -6148,7 +6146,7 @@
       <c r="A8" t="s">
         <v>27</v>
       </c>
-      <c r="B8" s="12">
+      <c r="B8" s="8">
         <v>0.1289</v>
       </c>
       <c r="C8" s="9">
@@ -6162,7 +6160,7 @@
       <c r="A9" t="s">
         <v>28</v>
       </c>
-      <c r="B9" s="12">
+      <c r="B9" s="8">
         <v>0.0202</v>
       </c>
       <c r="C9" s="9">
@@ -6176,7 +6174,7 @@
       <c r="A10" t="s">
         <v>29</v>
       </c>
-      <c r="B10" s="12">
+      <c r="B10" s="8">
         <v>0.141</v>
       </c>
       <c r="C10" s="9">
@@ -6190,7 +6188,7 @@
       <c r="A11" t="s">
         <v>30</v>
       </c>
-      <c r="B11" s="12">
+      <c r="B11" s="8">
         <v>0.047</v>
       </c>
       <c r="C11" s="9">
@@ -6204,7 +6202,7 @@
       <c r="A12" t="s">
         <v>31</v>
       </c>
-      <c r="B12" s="12">
+      <c r="B12" s="8">
         <v>0.092</v>
       </c>
       <c r="C12" s="9">
@@ -6218,7 +6216,7 @@
       <c r="A13" t="s">
         <v>32</v>
       </c>
-      <c r="B13" s="12">
+      <c r="B13" s="8">
         <v>0.1048</v>
       </c>
       <c r="C13" s="9">
@@ -6265,7 +6263,7 @@
       <c r="A18" t="s">
         <v>24</v>
       </c>
-      <c r="B18" s="12">
+      <c r="B18" s="8">
         <v>0.2247</v>
       </c>
       <c r="C18" s="9">
@@ -6279,7 +6277,7 @@
       <c r="A19" t="s">
         <v>25</v>
       </c>
-      <c r="B19" s="12">
+      <c r="B19" s="8">
         <v>0.1316</v>
       </c>
       <c r="C19" s="9">
@@ -6293,7 +6291,7 @@
       <c r="A20" t="s">
         <v>26</v>
       </c>
-      <c r="B20" s="12">
+      <c r="B20" s="8">
         <v>0.1439</v>
       </c>
       <c r="C20" s="9">
@@ -6307,7 +6305,7 @@
       <c r="A21" t="s">
         <v>27</v>
       </c>
-      <c r="B21" s="12">
+      <c r="B21" s="8">
         <v>0.093</v>
       </c>
       <c r="C21" s="9">
@@ -6321,7 +6319,7 @@
       <c r="A22" t="s">
         <v>28</v>
       </c>
-      <c r="B22" s="12">
+      <c r="B22" s="8">
         <v>0.0119</v>
       </c>
       <c r="C22" s="9">
@@ -6335,7 +6333,7 @@
       <c r="A23" t="s">
         <v>29</v>
       </c>
-      <c r="B23" s="12">
+      <c r="B23" s="8">
         <v>0.1316</v>
       </c>
       <c r="C23" s="9">
@@ -6349,7 +6347,7 @@
       <c r="A24" t="s">
         <v>30</v>
       </c>
-      <c r="B24" s="12">
+      <c r="B24" s="8">
         <v>0.0483</v>
       </c>
       <c r="C24" s="9">
@@ -6363,7 +6361,7 @@
       <c r="A25" t="s">
         <v>31</v>
       </c>
-      <c r="B25" s="12">
+      <c r="B25" s="8">
         <v>0.1122</v>
       </c>
       <c r="C25" s="9">
@@ -6377,7 +6375,7 @@
       <c r="A26" t="s">
         <v>32</v>
       </c>
-      <c r="B26" s="12">
+      <c r="B26" s="8">
         <v>0.1028</v>
       </c>
       <c r="C26" s="9">
@@ -6424,7 +6422,7 @@
       <c r="A31" t="s">
         <v>24</v>
       </c>
-      <c r="B31" s="12">
+      <c r="B31" s="8">
         <v>0.2022</v>
       </c>
       <c r="C31" s="9">
@@ -6438,7 +6436,7 @@
       <c r="A32" t="s">
         <v>25</v>
       </c>
-      <c r="B32" s="12">
+      <c r="B32" s="8">
         <v>0.1338</v>
       </c>
       <c r="C32" s="9">
@@ -6452,7 +6450,7 @@
       <c r="A33" t="s">
         <v>26</v>
       </c>
-      <c r="B33" s="12">
+      <c r="B33" s="8">
         <v>0.1242</v>
       </c>
       <c r="C33" s="9">
@@ -6466,7 +6464,7 @@
       <c r="A34" t="s">
         <v>27</v>
       </c>
-      <c r="B34" s="12">
+      <c r="B34" s="8">
         <v>0.1373</v>
       </c>
       <c r="C34" s="9">
@@ -6480,7 +6478,7 @@
       <c r="A35" t="s">
         <v>28</v>
       </c>
-      <c r="B35" s="12">
+      <c r="B35" s="8">
         <v>0.0406</v>
       </c>
       <c r="C35" s="9">
@@ -6494,7 +6492,7 @@
       <c r="A36" t="s">
         <v>29</v>
       </c>
-      <c r="B36" s="12">
+      <c r="B36" s="8">
         <v>0.1338</v>
       </c>
       <c r="C36" s="9">
@@ -6508,7 +6506,7 @@
       <c r="A37" t="s">
         <v>30</v>
       </c>
-      <c r="B37" s="12">
+      <c r="B37" s="8">
         <v>0.0333</v>
       </c>
       <c r="C37" s="9">
@@ -6522,7 +6520,7 @@
       <c r="A38" t="s">
         <v>31</v>
       </c>
-      <c r="B38" s="12">
+      <c r="B38" s="8">
         <v>0.1011</v>
       </c>
       <c r="C38" s="9">
@@ -6536,7 +6534,7 @@
       <c r="A39" t="s">
         <v>32</v>
       </c>
-      <c r="B39" s="12">
+      <c r="B39" s="8">
         <v>0.09379999999999999</v>
       </c>
       <c r="C39" s="9">

</xml_diff>